<commit_message>
Fill gaps from MacroStat export and NBU monetary survey
MacroStat (Andrey's sheet, exported to data/raw/manual, not committed): Gosstat
quarterly wages for the quarters the NBU API skips, monthly freight, registered
unemployment, gross external financing, debt payments and the payment schedule.
ms_oper.xlsx from the NBU adds monetary base, NBU certificates and NIR.
FREIGHT is now in million tonnes, the unit the data comes in.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RW4jPhKENmTAnc9qbN3YQ4
</commit_message>
<xml_diff>
--- a/data/history/history.xlsx
+++ b/data/history/history.xlsx
@@ -10,13 +10,14 @@
     <sheet name="ANCHORS_FACT" sheetId="1" r:id="rId1"/>
     <sheet name="SERIES_Q" sheetId="2" r:id="rId2"/>
     <sheet name="CATALOG" sheetId="3" r:id="rId3"/>
+    <sheet name="DEBT_SCHEDULE_Y" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="336">
   <si>
     <t>2015Q1</t>
   </si>
@@ -408,6 +409,27 @@
     <t>DEBT_UAH</t>
   </si>
   <si>
+    <t>REG_UNEMP</t>
+  </si>
+  <si>
+    <t>EXT_FIN_GROSS_USD</t>
+  </si>
+  <si>
+    <t>DEBT_PAY_UAH</t>
+  </si>
+  <si>
+    <t>DEBT_PAY_EXT_UAH</t>
+  </si>
+  <si>
+    <t>MONETARY_BASE</t>
+  </si>
+  <si>
+    <t>NBU_CD</t>
+  </si>
+  <si>
+    <t>NIR_USD</t>
+  </si>
+  <si>
     <t>WB_UNEMP</t>
   </si>
   <si>
@@ -519,7 +541,7 @@
     <t>Потребление электроэнергии</t>
   </si>
   <si>
-    <t>Грузооборот</t>
+    <t>Перевезення вантажів</t>
   </si>
   <si>
     <t>ВДС: сельское хозяйство</t>
@@ -678,6 +700,27 @@
     <t>Государственный и гарантированный долг</t>
   </si>
   <si>
+    <t>Зарегистрированные безработные, конец квартала</t>
+  </si>
+  <si>
+    <t>Валовое внешнее финансирование бюджета</t>
+  </si>
+  <si>
+    <t>Платежи по госдолгу (обслуживание + погашение)</t>
+  </si>
+  <si>
+    <t>Платежи по внешнему госдолгу</t>
+  </si>
+  <si>
+    <t>Денежная база</t>
+  </si>
+  <si>
+    <t>Депозитные сертификаты НБУ (избыток ликвидности)</t>
+  </si>
+  <si>
+    <t>Чистые международные резервы</t>
+  </si>
+  <si>
     <t>Безработица, модельная оценка МОТ</t>
   </si>
   <si>
@@ -717,7 +760,7 @@
     <t>млн кВт·ч</t>
   </si>
   <si>
-    <t>млн т·км</t>
+    <t>млн т</t>
   </si>
   <si>
     <t>% г/г</t>
@@ -741,6 +784,9 @@
     <t>НБУ API (Госстат, ОРС)</t>
   </si>
   <si>
+    <t>НБУ API (Госстат); пропуски из MacroStat</t>
+  </si>
+  <si>
     <t>НБУ API (платёжный баланс)</t>
   </si>
   <si>
@@ -750,7 +796,19 @@
     <t>Минфин (index.minfin.com.ua)</t>
   </si>
   <si>
-    <t>нет источника</t>
+    <t>Госстат (MacroStat, лист SectorIndexes M)</t>
+  </si>
+  <si>
+    <t>ГЦЗ (MacroStat, лист Salary)</t>
+  </si>
+  <si>
+    <t>MacroStat, лист Help (Минфин)</t>
+  </si>
+  <si>
+    <t>MacroStat, лист Debt (Минфин)</t>
+  </si>
+  <si>
+    <t>НБУ (ms_oper.xlsx)</t>
   </si>
   <si>
     <t>Всемирный банк</t>
@@ -801,7 +859,7 @@
     <t>Безработные / экономически активные 15–70; после 2021 нет данных</t>
   </si>
   <si>
-    <t>Средняя месячная зарплата, среднее за квартал</t>
+    <t>Средняя месячная зарплата, среднее за квартал; 2022–2023 и 2024Q3–Q4 из квартальных данных Госстата (лист Salary)</t>
   </si>
   <si>
     <t>Товары и услуги, кредит, сумма месяцев</t>
@@ -840,7 +898,7 @@
     <t>EG.USE.ELEC.KH.PC × население, годовое поровну на кварталы; до 2024, вся Украина</t>
   </si>
   <si>
-    <t>stat.gov.ua недоступен из облака; нужна выгрузка вручную</t>
+    <t>Перевезено грузов за месяц, сумма за квартал; ряд с 2018</t>
   </si>
   <si>
     <t>ea_gdp_ps_gv_add F_</t>
@@ -939,6 +997,15 @@
     <t>ED_GG, конец квартала</t>
   </si>
   <si>
+    <t>Строка TOTAL: 2022–2023 годовые суммы поровну на кварталы, с 2024 по месяцам</t>
+  </si>
+  <si>
+    <t>Сумма месяцев; с 2022</t>
+  </si>
+  <si>
+    <t>Всего минус внутренний долг, сумма месяцев; 2024Q3 включает реструктуризацию еврооблигаций</t>
+  </si>
+  <si>
     <t>SL.UEM.TOTL.ZS, годовое на все кварталы</t>
   </si>
   <si>
@@ -946,6 +1013,18 @@
   </si>
   <si>
     <t>series</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>domestic</t>
+  </si>
+  <si>
+    <t>external</t>
+  </si>
+  <si>
+    <t>year</t>
   </si>
 </sst>
 </file>
@@ -3569,11 +3648,41 @@
       <c r="AC17">
         <v>15260.13666666667</v>
       </c>
+      <c r="AD17">
+        <v>14620</v>
+      </c>
+      <c r="AE17">
+        <v>13723</v>
+      </c>
+      <c r="AF17">
+        <v>14619</v>
+      </c>
+      <c r="AG17">
+        <v>16477</v>
+      </c>
+      <c r="AH17">
+        <v>15435.96248</v>
+      </c>
+      <c r="AI17">
+        <v>17170.59728</v>
+      </c>
+      <c r="AJ17">
+        <v>18801.55322</v>
+      </c>
+      <c r="AK17">
+        <v>21180.30076</v>
+      </c>
       <c r="AL17">
         <v>18935.66666666667</v>
       </c>
       <c r="AM17">
         <v>21011</v>
+      </c>
+      <c r="AN17">
+        <v>22945.7511</v>
+      </c>
+      <c r="AO17">
+        <v>24153</v>
       </c>
       <c r="AP17">
         <v>23629</v>
@@ -4968,6 +5077,108 @@
     <row r="30" spans="1:48">
       <c r="A30" t="s">
         <v>77</v>
+      </c>
+      <c r="N30">
+        <v>150</v>
+      </c>
+      <c r="O30">
+        <v>154</v>
+      </c>
+      <c r="P30">
+        <v>159</v>
+      </c>
+      <c r="Q30">
+        <v>162</v>
+      </c>
+      <c r="R30">
+        <v>162</v>
+      </c>
+      <c r="S30">
+        <v>167</v>
+      </c>
+      <c r="T30">
+        <v>173</v>
+      </c>
+      <c r="U30">
+        <v>174</v>
+      </c>
+      <c r="V30">
+        <v>140.4</v>
+      </c>
+      <c r="W30">
+        <v>135</v>
+      </c>
+      <c r="X30">
+        <v>160</v>
+      </c>
+      <c r="Y30">
+        <v>164.7</v>
+      </c>
+      <c r="Z30">
+        <v>135.5</v>
+      </c>
+      <c r="AA30">
+        <v>152.4</v>
+      </c>
+      <c r="AB30">
+        <v>166.6</v>
+      </c>
+      <c r="AC30">
+        <v>166.8</v>
+      </c>
+      <c r="AD30">
+        <v>106.7</v>
+      </c>
+      <c r="AE30">
+        <v>63.4</v>
+      </c>
+      <c r="AF30">
+        <v>72</v>
+      </c>
+      <c r="AG30">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="AH30">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="AI30">
+        <v>77.8</v>
+      </c>
+      <c r="AJ30">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="AK30">
+        <v>92.8</v>
+      </c>
+      <c r="AL30">
+        <v>90.39999999999999</v>
+      </c>
+      <c r="AM30">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="AN30">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="AO30">
+        <v>89.7</v>
+      </c>
+      <c r="AP30">
+        <v>75.2</v>
+      </c>
+      <c r="AQ30">
+        <v>80.09999999999999</v>
+      </c>
+      <c r="AR30">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="AS30">
+        <v>83.5</v>
+      </c>
+      <c r="AT30">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="AU30">
+        <v>87.3532</v>
       </c>
     </row>
   </sheetData>
@@ -4977,7 +5188,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AV54"/>
+  <dimension ref="A1:AV61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:48">
@@ -12570,87 +12781,836 @@
         <v>130</v>
       </c>
       <c r="B54">
+        <v>506.791</v>
+      </c>
+      <c r="C54">
+        <v>443.938</v>
+      </c>
+      <c r="D54">
+        <v>407.383</v>
+      </c>
+      <c r="E54">
+        <v>490.775</v>
+      </c>
+      <c r="F54">
+        <v>467.5</v>
+      </c>
+      <c r="G54">
+        <v>388.931</v>
+      </c>
+      <c r="H54">
+        <v>341.511</v>
+      </c>
+      <c r="I54">
+        <v>390.787</v>
+      </c>
+      <c r="J54">
+        <v>406.757</v>
+      </c>
+      <c r="K54">
+        <v>330.2</v>
+      </c>
+      <c r="L54">
+        <v>302.966</v>
+      </c>
+      <c r="M54">
+        <v>354.394</v>
+      </c>
+      <c r="N54">
+        <v>366.881</v>
+      </c>
+      <c r="O54">
+        <v>303.9</v>
+      </c>
+      <c r="P54">
+        <v>287.1</v>
+      </c>
+      <c r="Q54">
+        <v>341.652</v>
+      </c>
+      <c r="R54">
+        <v>340.728</v>
+      </c>
+      <c r="S54">
+        <v>287.086</v>
+      </c>
+      <c r="T54">
+        <v>268.188</v>
+      </c>
+      <c r="U54">
+        <v>338.163</v>
+      </c>
+      <c r="V54">
+        <v>349.424</v>
+      </c>
+      <c r="W54">
+        <v>517.704</v>
+      </c>
+      <c r="X54">
+        <v>433.382</v>
+      </c>
+      <c r="Y54">
+        <v>459.2</v>
+      </c>
+      <c r="Z54">
+        <v>449.676</v>
+      </c>
+      <c r="AA54">
+        <v>344.788</v>
+      </c>
+      <c r="AB54">
+        <v>285.922</v>
+      </c>
+      <c r="AC54">
+        <v>294.968</v>
+      </c>
+      <c r="AD54">
+        <v>286.879</v>
+      </c>
+      <c r="AE54">
+        <v>316.448</v>
+      </c>
+      <c r="AF54">
+        <v>260.46</v>
+      </c>
+      <c r="AG54">
+        <v>186.508</v>
+      </c>
+      <c r="AH54">
+        <v>137.302</v>
+      </c>
+      <c r="AI54">
+        <v>113.376</v>
+      </c>
+      <c r="AJ54">
+        <v>103.252</v>
+      </c>
+      <c r="AK54">
+        <v>96.12</v>
+      </c>
+      <c r="AL54">
+        <v>118.468</v>
+      </c>
+      <c r="AM54">
+        <v>110.707</v>
+      </c>
+      <c r="AN54">
+        <v>102.749</v>
+      </c>
+      <c r="AO54">
+        <v>94.19</v>
+      </c>
+      <c r="AP54">
+        <v>101.358</v>
+      </c>
+      <c r="AQ54">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="AR54">
+        <v>92.8</v>
+      </c>
+      <c r="AS54">
+        <v>88.3</v>
+      </c>
+      <c r="AT54">
+        <v>96.5</v>
+      </c>
+      <c r="AU54">
+        <v>93.09999999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:48">
+      <c r="A55" t="s">
+        <v>131</v>
+      </c>
+      <c r="AD55">
+        <v>7773.75</v>
+      </c>
+      <c r="AE55">
+        <v>7773.75</v>
+      </c>
+      <c r="AF55">
+        <v>7773.75</v>
+      </c>
+      <c r="AG55">
+        <v>7773.75</v>
+      </c>
+      <c r="AH55">
+        <v>10619.75</v>
+      </c>
+      <c r="AI55">
+        <v>10619.75</v>
+      </c>
+      <c r="AJ55">
+        <v>10619.75</v>
+      </c>
+      <c r="AK55">
+        <v>10619.75</v>
+      </c>
+      <c r="AL55">
+        <v>10340.7</v>
+      </c>
+      <c r="AM55">
+        <v>3647.5</v>
+      </c>
+      <c r="AN55">
+        <v>10718.9</v>
+      </c>
+      <c r="AO55">
+        <v>18368.8</v>
+      </c>
+      <c r="AP55">
+        <v>10360.6</v>
+      </c>
+      <c r="AQ55">
+        <v>12364.4</v>
+      </c>
+      <c r="AR55">
+        <v>10080.8</v>
+      </c>
+      <c r="AS55">
+        <v>18606.3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:48">
+      <c r="A56" t="s">
+        <v>132</v>
+      </c>
+      <c r="AD56">
+        <v>135360</v>
+      </c>
+      <c r="AE56">
+        <v>166230</v>
+      </c>
+      <c r="AF56">
+        <v>109130</v>
+      </c>
+      <c r="AG56">
+        <v>195860</v>
+      </c>
+      <c r="AH56">
+        <v>122010</v>
+      </c>
+      <c r="AI56">
+        <v>240930</v>
+      </c>
+      <c r="AJ56">
+        <v>159580</v>
+      </c>
+      <c r="AK56">
+        <v>162320</v>
+      </c>
+      <c r="AL56">
+        <v>159370</v>
+      </c>
+      <c r="AM56">
+        <v>232560</v>
+      </c>
+      <c r="AN56">
+        <v>769810</v>
+      </c>
+      <c r="AO56">
+        <v>270590</v>
+      </c>
+      <c r="AP56">
+        <v>218400</v>
+      </c>
+      <c r="AQ56">
+        <v>283860</v>
+      </c>
+      <c r="AR56">
+        <v>194960</v>
+      </c>
+      <c r="AS56">
+        <v>259140</v>
+      </c>
+      <c r="AT56">
+        <v>204450</v>
+      </c>
+      <c r="AU56">
+        <v>268530</v>
+      </c>
+      <c r="AV56">
+        <v>226770</v>
+      </c>
+    </row>
+    <row r="57" spans="1:48">
+      <c r="A57" t="s">
+        <v>133</v>
+      </c>
+      <c r="AD57">
+        <v>28580.00000000001</v>
+      </c>
+      <c r="AE57">
+        <v>22239.99999999999</v>
+      </c>
+      <c r="AF57">
+        <v>11640</v>
+      </c>
+      <c r="AG57">
+        <v>24300</v>
+      </c>
+      <c r="AH57">
+        <v>25180</v>
+      </c>
+      <c r="AI57">
+        <v>19380</v>
+      </c>
+      <c r="AJ57">
+        <v>38840</v>
+      </c>
+      <c r="AK57">
+        <v>31919.99999999999</v>
+      </c>
+      <c r="AL57">
+        <v>44650</v>
+      </c>
+      <c r="AM57">
+        <v>63090.00000000001</v>
+      </c>
+      <c r="AN57">
+        <v>667170</v>
+      </c>
+      <c r="AO57">
+        <v>58570.00000000003</v>
+      </c>
+      <c r="AP57">
+        <v>55650</v>
+      </c>
+      <c r="AQ57">
+        <v>65390.00000000001</v>
+      </c>
+      <c r="AR57">
+        <v>42780.00000000001</v>
+      </c>
+      <c r="AS57">
+        <v>50170</v>
+      </c>
+      <c r="AT57">
+        <v>59350</v>
+      </c>
+      <c r="AU57">
+        <v>56300</v>
+      </c>
+      <c r="AV57">
+        <v>68460</v>
+      </c>
+    </row>
+    <row r="58" spans="1:48">
+      <c r="A58" t="s">
+        <v>134</v>
+      </c>
+      <c r="B58">
+        <v>331991.32964555</v>
+      </c>
+      <c r="C58">
+        <v>330379.08319171</v>
+      </c>
+      <c r="D58">
+        <v>321206.65875189</v>
+      </c>
+      <c r="E58">
+        <v>335999.64216584</v>
+      </c>
+      <c r="F58">
+        <v>327219.86727566</v>
+      </c>
+      <c r="G58">
+        <v>352649.13827149</v>
+      </c>
+      <c r="H58">
+        <v>355191.68210861</v>
+      </c>
+      <c r="I58">
+        <v>381575.48956979</v>
+      </c>
+      <c r="J58">
+        <v>356913.89151764</v>
+      </c>
+      <c r="K58">
+        <v>381757.06465185</v>
+      </c>
+      <c r="L58">
+        <v>373400.46175206</v>
+      </c>
+      <c r="M58">
+        <v>399056.72668439</v>
+      </c>
+      <c r="N58">
+        <v>393232.21817462</v>
+      </c>
+      <c r="O58">
+        <v>419954.33327615</v>
+      </c>
+      <c r="P58">
+        <v>424356.80395804</v>
+      </c>
+      <c r="Q58">
+        <v>435797.70191339</v>
+      </c>
+      <c r="R58">
+        <v>423715.0614647</v>
+      </c>
+      <c r="S58">
+        <v>445084.67264794</v>
+      </c>
+      <c r="T58">
+        <v>441010.11253476</v>
+      </c>
+      <c r="U58">
+        <v>477490.55573389</v>
+      </c>
+      <c r="V58">
+        <v>481846.77134785</v>
+      </c>
+      <c r="W58">
+        <v>532651.87541945</v>
+      </c>
+      <c r="X58">
+        <v>567877.30037951</v>
+      </c>
+      <c r="Y58">
+        <v>595986.1001978</v>
+      </c>
+      <c r="Z58">
+        <v>608662.34515793</v>
+      </c>
+      <c r="AA58">
+        <v>645019.00763999</v>
+      </c>
+      <c r="AB58">
+        <v>644383.72109489</v>
+      </c>
+      <c r="AC58">
+        <v>662498.99473475</v>
+      </c>
+      <c r="AD58">
+        <v>732841.50363819</v>
+      </c>
+      <c r="AE58">
+        <v>729369.66297768</v>
+      </c>
+      <c r="AF58">
+        <v>740492.30557939</v>
+      </c>
+      <c r="AG58">
+        <v>792536.81339446</v>
+      </c>
+      <c r="AH58">
+        <v>863753.46562943</v>
+      </c>
+      <c r="AI58">
+        <v>907458.1948201701</v>
+      </c>
+      <c r="AJ58">
+        <v>927391.94967376</v>
+      </c>
+      <c r="AK58">
+        <v>976939.94212763</v>
+      </c>
+      <c r="AL58">
+        <v>1007051.47569272</v>
+      </c>
+      <c r="AM58">
+        <v>1079531.0195509</v>
+      </c>
+      <c r="AN58">
+        <v>1049356.92328563</v>
+      </c>
+      <c r="AO58">
+        <v>1052112.61405579</v>
+      </c>
+      <c r="AP58">
+        <v>1011542.6223512</v>
+      </c>
+      <c r="AQ58">
+        <v>1098856.59631834</v>
+      </c>
+      <c r="AR58">
+        <v>1125575.58585739</v>
+      </c>
+      <c r="AS58">
+        <v>1174525.58851348</v>
+      </c>
+      <c r="AT58">
+        <v>1193658.25862318</v>
+      </c>
+      <c r="AU58">
+        <v>1247325.053641</v>
+      </c>
+    </row>
+    <row r="59" spans="1:48">
+      <c r="A59" t="s">
+        <v>135</v>
+      </c>
+      <c r="B59">
+        <v>14180.29874873</v>
+      </c>
+      <c r="C59">
+        <v>39501.93416776</v>
+      </c>
+      <c r="D59">
+        <v>47571.55087035</v>
+      </c>
+      <c r="E59">
+        <v>89844.97663238</v>
+      </c>
+      <c r="F59">
+        <v>63538.38582873</v>
+      </c>
+      <c r="G59">
+        <v>49732.05064097</v>
+      </c>
+      <c r="H59">
+        <v>35423.43416155</v>
+      </c>
+      <c r="I59">
+        <v>68167.0072137</v>
+      </c>
+      <c r="J59">
+        <v>65490.83320005</v>
+      </c>
+      <c r="K59">
+        <v>53652.67931436</v>
+      </c>
+      <c r="L59">
+        <v>36836.09165695</v>
+      </c>
+      <c r="M59">
+        <v>67189.60473016</v>
+      </c>
+      <c r="N59">
+        <v>59667.37809696</v>
+      </c>
+      <c r="O59">
+        <v>63478.64471546</v>
+      </c>
+      <c r="P59">
+        <v>28607.54607179</v>
+      </c>
+      <c r="Q59">
+        <v>62075.8384136</v>
+      </c>
+      <c r="R59">
+        <v>58049.6611917</v>
+      </c>
+      <c r="S59">
+        <v>45459.69561334</v>
+      </c>
+      <c r="T59">
+        <v>60044.44435013</v>
+      </c>
+      <c r="U59">
+        <v>152212.06477884</v>
+      </c>
+      <c r="V59">
+        <v>115509.40197648</v>
+      </c>
+      <c r="W59">
+        <v>104872.46521549</v>
+      </c>
+      <c r="X59">
+        <v>122672.06716853</v>
+      </c>
+      <c r="Y59">
+        <v>163645.66606426</v>
+      </c>
+      <c r="Z59">
+        <v>143534.66881938</v>
+      </c>
+      <c r="AA59">
+        <v>157125.04515888</v>
+      </c>
+      <c r="AB59">
+        <v>144499.37619341</v>
+      </c>
+      <c r="AC59">
+        <v>212925.63327876</v>
+      </c>
+      <c r="AD59">
+        <v>141837.96578374</v>
+      </c>
+      <c r="AE59">
+        <v>189364.2508443</v>
+      </c>
+      <c r="AF59">
+        <v>257720.29759812</v>
+      </c>
+      <c r="AG59">
+        <v>457463.80223976</v>
+      </c>
+      <c r="AH59">
+        <v>352886.22769296</v>
+      </c>
+      <c r="AI59">
+        <v>478869.80173876</v>
+      </c>
+      <c r="AJ59">
+        <v>514464.4012031</v>
+      </c>
+      <c r="AK59">
+        <v>621666.50101772</v>
+      </c>
+      <c r="AL59">
+        <v>549419.3057422</v>
+      </c>
+      <c r="AM59">
+        <v>510386.37196891</v>
+      </c>
+      <c r="AN59">
+        <v>467542.13961082</v>
+      </c>
+      <c r="AO59">
+        <v>548911.03139254</v>
+      </c>
+      <c r="AP59">
+        <v>541769.36949879</v>
+      </c>
+      <c r="AQ59">
+        <v>542208.96866842</v>
+      </c>
+      <c r="AR59">
+        <v>499858.00027585</v>
+      </c>
+      <c r="AS59">
+        <v>775684.5196034</v>
+      </c>
+      <c r="AT59">
+        <v>573092.60091902</v>
+      </c>
+      <c r="AU59">
+        <v>663296.3742342</v>
+      </c>
+    </row>
+    <row r="60" spans="1:48">
+      <c r="A60" t="s">
+        <v>136</v>
+      </c>
+      <c r="B60">
+        <v>29.07</v>
+      </c>
+      <c r="C60">
+        <v>524.5434</v>
+      </c>
+      <c r="D60">
+        <v>1288.1212</v>
+      </c>
+      <c r="E60">
+        <v>1335.8312</v>
+      </c>
+      <c r="F60">
+        <v>1032.5061</v>
+      </c>
+      <c r="G60">
+        <v>3209.525252605416</v>
+      </c>
+      <c r="H60">
+        <v>3840.346357126271</v>
+      </c>
+      <c r="I60">
+        <v>4224.247727003089</v>
+      </c>
+      <c r="J60">
+        <v>3702.8722502327</v>
+      </c>
+      <c r="K60">
+        <v>5230.287941602684</v>
+      </c>
+      <c r="L60">
+        <v>6068.341530395468</v>
+      </c>
+      <c r="M60">
+        <v>6671.83941593941</v>
+      </c>
+      <c r="N60">
+        <v>6342.163199703901</v>
+      </c>
+      <c r="O60">
+        <v>7036.94505252085</v>
+      </c>
+      <c r="P60">
+        <v>6302.5848999956</v>
+      </c>
+      <c r="Q60">
+        <v>9644.363417352479</v>
+      </c>
+      <c r="R60">
+        <v>9993.071022464501</v>
+      </c>
+      <c r="S60">
+        <v>10500.72307913855</v>
+      </c>
+      <c r="T60">
+        <v>12054.5005159014</v>
+      </c>
+      <c r="U60">
+        <v>15784.50174752007</v>
+      </c>
+      <c r="V60">
+        <v>16067.9096603352</v>
+      </c>
+      <c r="W60">
+        <v>17495.1090329364</v>
+      </c>
+      <c r="X60">
+        <v>15795.58273911649</v>
+      </c>
+      <c r="Y60">
+        <v>18114.41681427242</v>
+      </c>
+      <c r="Z60">
+        <v>16744.4244982683</v>
+      </c>
+      <c r="AA60">
+        <v>17976.5273513692</v>
+      </c>
+      <c r="AB60">
+        <v>19095.456478546</v>
+      </c>
+      <c r="AC60">
+        <v>20767.157481153</v>
+      </c>
+      <c r="AD60">
+        <v>17569.9103259394</v>
+      </c>
+      <c r="AE60">
+        <v>12951.0523989499</v>
+      </c>
+      <c r="AF60">
+        <v>15183.6405010308</v>
+      </c>
+      <c r="AG60">
+        <v>18321.5104002509</v>
+      </c>
+      <c r="AH60">
+        <v>22430.285836947</v>
+      </c>
+      <c r="AI60">
+        <v>26365.3557825058</v>
+      </c>
+      <c r="AJ60">
+        <v>28212.813641948</v>
+      </c>
+      <c r="AK60">
+        <v>28381.4293816899</v>
+      </c>
+      <c r="AL60">
+        <v>31763.3347116023</v>
+      </c>
+      <c r="AM60">
+        <v>26298.5585579431</v>
+      </c>
+      <c r="AN60">
+        <v>25547.4369360588</v>
+      </c>
+      <c r="AO60">
+        <v>29101.6834874098</v>
+      </c>
+      <c r="AP60">
+        <v>27949.6142433875</v>
+      </c>
+      <c r="AQ60">
+        <v>30742.9611376797</v>
+      </c>
+      <c r="AR60">
+        <v>32306.001452845</v>
+      </c>
+      <c r="AS60">
+        <v>43327.2324435414</v>
+      </c>
+      <c r="AT60">
+        <v>37171.9912995195</v>
+      </c>
+      <c r="AU60">
+        <v>36949.76002921</v>
+      </c>
+    </row>
+    <row r="61" spans="1:48">
+      <c r="A61" t="s">
+        <v>137</v>
+      </c>
+      <c r="B61">
         <v>9.140000000000001</v>
       </c>
-      <c r="C54">
+      <c r="C61">
         <v>9.140000000000001</v>
       </c>
-      <c r="D54">
+      <c r="D61">
         <v>9.140000000000001</v>
       </c>
-      <c r="E54">
+      <c r="E61">
         <v>9.140000000000001</v>
       </c>
-      <c r="F54">
+      <c r="F61">
         <v>9.35</v>
       </c>
-      <c r="G54">
+      <c r="G61">
         <v>9.35</v>
       </c>
-      <c r="H54">
+      <c r="H61">
         <v>9.35</v>
       </c>
-      <c r="I54">
+      <c r="I61">
         <v>9.35</v>
       </c>
-      <c r="J54">
+      <c r="J61">
         <v>9.5</v>
       </c>
-      <c r="K54">
+      <c r="K61">
         <v>9.5</v>
       </c>
-      <c r="L54">
+      <c r="L61">
         <v>9.5</v>
       </c>
-      <c r="M54">
+      <c r="M61">
         <v>9.5</v>
       </c>
-      <c r="N54">
+      <c r="N61">
         <v>8.798999999999999</v>
       </c>
-      <c r="O54">
+      <c r="O61">
         <v>8.798999999999999</v>
       </c>
-      <c r="P54">
+      <c r="P61">
         <v>8.798999999999999</v>
       </c>
-      <c r="Q54">
+      <c r="Q61">
         <v>8.798999999999999</v>
       </c>
-      <c r="R54">
+      <c r="R61">
         <v>8.194000000000001</v>
       </c>
-      <c r="S54">
+      <c r="S61">
         <v>8.194000000000001</v>
       </c>
-      <c r="T54">
+      <c r="T61">
         <v>8.194000000000001</v>
       </c>
-      <c r="U54">
+      <c r="U61">
         <v>8.194000000000001</v>
       </c>
-      <c r="V54">
+      <c r="V61">
         <v>9.475</v>
       </c>
-      <c r="W54">
+      <c r="W61">
         <v>9.475</v>
       </c>
-      <c r="X54">
+      <c r="X61">
         <v>9.475</v>
       </c>
-      <c r="Y54">
+      <c r="Y61">
         <v>9.475</v>
       </c>
-      <c r="Z54">
+      <c r="Z61">
         <v>9.834</v>
       </c>
-      <c r="AA54">
+      <c r="AA61">
         <v>9.834</v>
       </c>
-      <c r="AB54">
+      <c r="AB61">
         <v>9.834</v>
       </c>
-      <c r="AC54">
+      <c r="AC61">
         <v>9.834</v>
       </c>
     </row>
@@ -12661,7 +13621,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -12669,28 +13629,28 @@
         <v>48</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C1" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="D1" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E1" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="F1" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="G1" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="H1" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="I1" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -12698,16 +13658,16 @@
         <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C2" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="D2" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E2" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="F2" t="s">
         <v>0</v>
@@ -12719,7 +13679,7 @@
         <v>46</v>
       </c>
       <c r="I2" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -12727,16 +13687,16 @@
         <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C3" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="D3" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E3" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="F3" t="s">
         <v>0</v>
@@ -12748,7 +13708,7 @@
         <v>46</v>
       </c>
       <c r="I3" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -12756,16 +13716,16 @@
         <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C4" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="D4" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E4" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="F4" t="s">
         <v>0</v>
@@ -12777,7 +13737,7 @@
         <v>46</v>
       </c>
       <c r="I4" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -12785,16 +13745,16 @@
         <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C5" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D5" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E5" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
@@ -12806,7 +13766,7 @@
         <v>46</v>
       </c>
       <c r="I5" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -12814,16 +13774,16 @@
         <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="D6" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="E6" t="s">
-        <v>250</v>
+        <v>269</v>
       </c>
       <c r="F6" t="s">
         <v>0</v>
@@ -12835,7 +13795,7 @@
         <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -12843,16 +13803,16 @@
         <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C7" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="D7" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E7" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
       <c r="F7" t="s">
         <v>0</v>
@@ -12864,7 +13824,7 @@
         <v>47</v>
       </c>
       <c r="I7" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -12872,16 +13832,16 @@
         <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C8" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="D8" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E8" t="s">
-        <v>252</v>
+        <v>271</v>
       </c>
       <c r="F8" t="s">
         <v>0</v>
@@ -12893,7 +13853,7 @@
         <v>46</v>
       </c>
       <c r="I8" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -12901,16 +13861,16 @@
         <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C9" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="D9" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="E9" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="F9" t="s">
         <v>0</v>
@@ -12922,7 +13882,7 @@
         <v>48</v>
       </c>
       <c r="I9" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -12930,16 +13890,16 @@
         <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C10" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="D10" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="E10" t="s">
-        <v>254</v>
+        <v>273</v>
       </c>
       <c r="F10" t="s">
         <v>0</v>
@@ -12951,7 +13911,7 @@
         <v>48</v>
       </c>
       <c r="I10" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -12959,16 +13919,16 @@
         <v>58</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C11" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D11" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E11" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="F11" t="s">
         <v>0</v>
@@ -12980,7 +13940,7 @@
         <v>48</v>
       </c>
       <c r="I11" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -12988,16 +13948,16 @@
         <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="C12" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D12" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E12" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
       <c r="F12" t="s">
         <v>0</v>
@@ -13009,7 +13969,7 @@
         <v>46</v>
       </c>
       <c r="I12" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -13017,16 +13977,16 @@
         <v>60</v>
       </c>
       <c r="B13" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C13" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D13" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E13" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="F13" t="s">
         <v>0</v>
@@ -13038,7 +13998,7 @@
         <v>46</v>
       </c>
       <c r="I13" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -13046,16 +14006,16 @@
         <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C14" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="D14" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="E14" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
       <c r="F14" t="s">
         <v>0</v>
@@ -13067,7 +14027,7 @@
         <v>44</v>
       </c>
       <c r="I14" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -13075,16 +14035,16 @@
         <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C15" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="D15" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="E15" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="F15" t="s">
         <v>0</v>
@@ -13096,7 +14056,7 @@
         <v>28</v>
       </c>
       <c r="I15" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -13104,16 +14064,16 @@
         <v>63</v>
       </c>
       <c r="B16" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C16" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D16" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="E16" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
       <c r="F16" t="s">
         <v>0</v>
@@ -13125,7 +14085,7 @@
         <v>28</v>
       </c>
       <c r="I16" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -13133,16 +14093,16 @@
         <v>64</v>
       </c>
       <c r="B17" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C17" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="D17" t="s">
-        <v>235</v>
+        <v>255</v>
       </c>
       <c r="E17" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="F17" t="s">
         <v>0</v>
@@ -13151,10 +14111,10 @@
         <v>45</v>
       </c>
       <c r="H17">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="I17" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -13162,16 +14122,16 @@
         <v>65</v>
       </c>
       <c r="B18" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="C18" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D18" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E18" t="s">
-        <v>262</v>
+        <v>281</v>
       </c>
       <c r="F18" t="s">
         <v>0</v>
@@ -13183,7 +14143,7 @@
         <v>46</v>
       </c>
       <c r="I18" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -13191,16 +14151,16 @@
         <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C19" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D19" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E19" t="s">
-        <v>263</v>
+        <v>282</v>
       </c>
       <c r="F19" t="s">
         <v>0</v>
@@ -13212,7 +14172,7 @@
         <v>46</v>
       </c>
       <c r="I19" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -13220,16 +14180,16 @@
         <v>67</v>
       </c>
       <c r="B20" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C20" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D20" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="E20" t="s">
-        <v>264</v>
+        <v>283</v>
       </c>
       <c r="F20" t="s">
         <v>0</v>
@@ -13241,7 +14201,7 @@
         <v>46</v>
       </c>
       <c r="I20" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -13249,16 +14209,16 @@
         <v>68</v>
       </c>
       <c r="B21" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C21" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D21" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E21" t="s">
-        <v>265</v>
+        <v>284</v>
       </c>
       <c r="F21" t="s">
         <v>0</v>
@@ -13270,7 +14230,7 @@
         <v>47</v>
       </c>
       <c r="I21" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -13278,16 +14238,16 @@
         <v>69</v>
       </c>
       <c r="B22" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C22" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D22" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E22" t="s">
-        <v>266</v>
+        <v>285</v>
       </c>
       <c r="F22" t="s">
         <v>0</v>
@@ -13299,7 +14259,7 @@
         <v>46</v>
       </c>
       <c r="I22" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -13307,16 +14267,16 @@
         <v>70</v>
       </c>
       <c r="B23" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C23" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D23" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="E23" t="s">
-        <v>267</v>
+        <v>286</v>
       </c>
       <c r="F23" t="s">
         <v>0</v>
@@ -13328,7 +14288,7 @@
         <v>28</v>
       </c>
       <c r="I23" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -13336,16 +14296,16 @@
         <v>71</v>
       </c>
       <c r="B24" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C24" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D24" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="E24" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="F24" t="s">
         <v>0</v>
@@ -13357,7 +14317,7 @@
         <v>46</v>
       </c>
       <c r="I24" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -13365,22 +14325,22 @@
         <v>72</v>
       </c>
       <c r="B25" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C25" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D25" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="E25" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="I25" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -13388,16 +14348,16 @@
         <v>73</v>
       </c>
       <c r="B26" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C26" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D26" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E26" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="F26" t="s">
         <v>0</v>
@@ -13409,7 +14369,7 @@
         <v>46</v>
       </c>
       <c r="I26" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -13417,22 +14377,22 @@
         <v>74</v>
       </c>
       <c r="B27" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C27" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D27" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="E27" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
       <c r="H27">
         <v>0</v>
       </c>
       <c r="I27" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -13440,16 +14400,16 @@
         <v>75</v>
       </c>
       <c r="B28" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="D28" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="E28" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="F28" t="s">
         <v>0</v>
@@ -13461,7 +14421,7 @@
         <v>46</v>
       </c>
       <c r="I28" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -13469,16 +14429,16 @@
         <v>76</v>
       </c>
       <c r="B29" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C29" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="D29" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="E29" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
       <c r="F29" t="s">
         <v>0</v>
@@ -13490,7 +14450,7 @@
         <v>40</v>
       </c>
       <c r="I29" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -13498,22 +14458,28 @@
         <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C30" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="D30" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="E30" t="s">
-        <v>274</v>
+        <v>293</v>
+      </c>
+      <c r="F30" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" t="s">
+        <v>45</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I30" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -13521,16 +14487,16 @@
         <v>78</v>
       </c>
       <c r="B31" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C31" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D31" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E31" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F31" t="s">
         <v>0</v>
@@ -13542,7 +14508,7 @@
         <v>46</v>
       </c>
       <c r="I31" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -13550,16 +14516,16 @@
         <v>79</v>
       </c>
       <c r="B32" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C32" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D32" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E32" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F32" t="s">
         <v>0</v>
@@ -13571,7 +14537,7 @@
         <v>46</v>
       </c>
       <c r="I32" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -13579,16 +14545,16 @@
         <v>80</v>
       </c>
       <c r="B33" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C33" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D33" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E33" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F33" t="s">
         <v>0</v>
@@ -13600,7 +14566,7 @@
         <v>46</v>
       </c>
       <c r="I33" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -13608,16 +14574,16 @@
         <v>81</v>
       </c>
       <c r="B34" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C34" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D34" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E34" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F34" t="s">
         <v>0</v>
@@ -13629,7 +14595,7 @@
         <v>46</v>
       </c>
       <c r="I34" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -13637,16 +14603,16 @@
         <v>82</v>
       </c>
       <c r="B35" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C35" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D35" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E35" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F35" t="s">
         <v>0</v>
@@ -13658,7 +14624,7 @@
         <v>46</v>
       </c>
       <c r="I35" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -13666,16 +14632,16 @@
         <v>83</v>
       </c>
       <c r="B36" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C36" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D36" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E36" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F36" t="s">
         <v>0</v>
@@ -13687,7 +14653,7 @@
         <v>46</v>
       </c>
       <c r="I36" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -13695,16 +14661,16 @@
         <v>84</v>
       </c>
       <c r="B37" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C37" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D37" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E37" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F37" t="s">
         <v>0</v>
@@ -13716,7 +14682,7 @@
         <v>46</v>
       </c>
       <c r="I37" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -13724,16 +14690,16 @@
         <v>85</v>
       </c>
       <c r="B38" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="C38" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D38" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E38" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F38" t="s">
         <v>0</v>
@@ -13745,7 +14711,7 @@
         <v>46</v>
       </c>
       <c r="I38" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -13753,16 +14719,16 @@
         <v>86</v>
       </c>
       <c r="B39" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C39" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D39" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E39" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F39" t="s">
         <v>0</v>
@@ -13774,7 +14740,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -13782,16 +14748,16 @@
         <v>87</v>
       </c>
       <c r="B40" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="C40" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D40" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E40" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F40" t="s">
         <v>0</v>
@@ -13803,7 +14769,7 @@
         <v>46</v>
       </c>
       <c r="I40" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -13811,16 +14777,16 @@
         <v>88</v>
       </c>
       <c r="B41" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C41" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D41" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E41" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F41" t="s">
         <v>0</v>
@@ -13832,7 +14798,7 @@
         <v>46</v>
       </c>
       <c r="I41" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -13840,16 +14806,16 @@
         <v>89</v>
       </c>
       <c r="B42" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C42" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D42" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E42" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F42" t="s">
         <v>0</v>
@@ -13861,7 +14827,7 @@
         <v>46</v>
       </c>
       <c r="I42" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -13869,16 +14835,16 @@
         <v>90</v>
       </c>
       <c r="B43" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C43" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D43" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E43" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F43" t="s">
         <v>0</v>
@@ -13890,7 +14856,7 @@
         <v>46</v>
       </c>
       <c r="I43" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -13898,16 +14864,16 @@
         <v>91</v>
       </c>
       <c r="B44" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C44" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D44" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E44" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F44" t="s">
         <v>0</v>
@@ -13919,7 +14885,7 @@
         <v>46</v>
       </c>
       <c r="I44" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -13927,16 +14893,16 @@
         <v>92</v>
       </c>
       <c r="B45" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C45" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D45" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E45" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F45" t="s">
         <v>0</v>
@@ -13948,7 +14914,7 @@
         <v>46</v>
       </c>
       <c r="I45" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -13956,16 +14922,16 @@
         <v>93</v>
       </c>
       <c r="B46" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C46" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D46" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E46" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F46" t="s">
         <v>0</v>
@@ -13977,7 +14943,7 @@
         <v>46</v>
       </c>
       <c r="I46" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -13985,16 +14951,16 @@
         <v>94</v>
       </c>
       <c r="B47" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C47" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D47" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E47" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="F47" t="s">
         <v>0</v>
@@ -14006,7 +14972,7 @@
         <v>46</v>
       </c>
       <c r="I47" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -14014,16 +14980,16 @@
         <v>95</v>
       </c>
       <c r="B48" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D48" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E48" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="F48" t="s">
         <v>0</v>
@@ -14035,7 +15001,7 @@
         <v>46</v>
       </c>
       <c r="I48" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -14043,16 +15009,16 @@
         <v>96</v>
       </c>
       <c r="B49" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C49" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D49" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E49" t="s">
-        <v>277</v>
+        <v>296</v>
       </c>
       <c r="F49" t="s">
         <v>0</v>
@@ -14064,7 +15030,7 @@
         <v>46</v>
       </c>
       <c r="I49" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -14072,16 +15038,16 @@
         <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C50" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D50" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E50" t="s">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="F50" t="s">
         <v>0</v>
@@ -14093,7 +15059,7 @@
         <v>46</v>
       </c>
       <c r="I50" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -14101,16 +15067,16 @@
         <v>98</v>
       </c>
       <c r="B51" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C51" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D51" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E51" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="F51" t="s">
         <v>0</v>
@@ -14122,7 +15088,7 @@
         <v>46</v>
       </c>
       <c r="I51" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -14130,16 +15096,16 @@
         <v>99</v>
       </c>
       <c r="B52" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C52" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D52" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E52" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="F52" t="s">
         <v>0</v>
@@ -14151,7 +15117,7 @@
         <v>46</v>
       </c>
       <c r="I52" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -14159,16 +15125,16 @@
         <v>100</v>
       </c>
       <c r="B53" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C53" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D53" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E53" t="s">
-        <v>281</v>
+        <v>300</v>
       </c>
       <c r="F53" t="s">
         <v>0</v>
@@ -14180,7 +15146,7 @@
         <v>46</v>
       </c>
       <c r="I53" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -14188,16 +15154,16 @@
         <v>101</v>
       </c>
       <c r="B54" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C54" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D54" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E54" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="F54" t="s">
         <v>0</v>
@@ -14209,7 +15175,7 @@
         <v>46</v>
       </c>
       <c r="I54" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -14217,16 +15183,16 @@
         <v>102</v>
       </c>
       <c r="B55" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C55" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D55" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E55" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="F55" t="s">
         <v>0</v>
@@ -14238,7 +15204,7 @@
         <v>46</v>
       </c>
       <c r="I55" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -14246,16 +15212,16 @@
         <v>103</v>
       </c>
       <c r="B56" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="C56" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D56" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E56" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="F56" t="s">
         <v>0</v>
@@ -14267,7 +15233,7 @@
         <v>46</v>
       </c>
       <c r="I56" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -14275,16 +15241,16 @@
         <v>104</v>
       </c>
       <c r="B57" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C57" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D57" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E57" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
       <c r="F57" t="s">
         <v>0</v>
@@ -14296,7 +15262,7 @@
         <v>46</v>
       </c>
       <c r="I57" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -14304,16 +15270,16 @@
         <v>105</v>
       </c>
       <c r="B58" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C58" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D58" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E58" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
       <c r="F58" t="s">
         <v>0</v>
@@ -14325,7 +15291,7 @@
         <v>46</v>
       </c>
       <c r="I58" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -14333,16 +15299,16 @@
         <v>106</v>
       </c>
       <c r="B59" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C59" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D59" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E59" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="F59" t="s">
         <v>0</v>
@@ -14354,7 +15320,7 @@
         <v>46</v>
       </c>
       <c r="I59" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -14362,16 +15328,16 @@
         <v>107</v>
       </c>
       <c r="B60" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="C60" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D60" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E60" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
       <c r="F60" t="s">
         <v>0</v>
@@ -14383,7 +15349,7 @@
         <v>46</v>
       </c>
       <c r="I60" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -14391,16 +15357,16 @@
         <v>108</v>
       </c>
       <c r="B61" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C61" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D61" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E61" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="F61" t="s">
         <v>0</v>
@@ -14412,7 +15378,7 @@
         <v>46</v>
       </c>
       <c r="I61" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -14420,16 +15386,16 @@
         <v>109</v>
       </c>
       <c r="B62" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C62" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D62" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E62" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="F62" t="s">
         <v>0</v>
@@ -14441,7 +15407,7 @@
         <v>47</v>
       </c>
       <c r="I62" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -14449,16 +15415,16 @@
         <v>110</v>
       </c>
       <c r="B63" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C63" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D63" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E63" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="F63" t="s">
         <v>0</v>
@@ -14470,7 +15436,7 @@
         <v>47</v>
       </c>
       <c r="I63" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -14478,16 +15444,16 @@
         <v>111</v>
       </c>
       <c r="B64" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C64" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D64" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E64" t="s">
-        <v>292</v>
+        <v>311</v>
       </c>
       <c r="F64" t="s">
         <v>0</v>
@@ -14499,7 +15465,7 @@
         <v>46</v>
       </c>
       <c r="I64" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -14507,16 +15473,16 @@
         <v>112</v>
       </c>
       <c r="B65" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C65" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D65" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E65" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
       <c r="F65" t="s">
         <v>0</v>
@@ -14528,7 +15494,7 @@
         <v>46</v>
       </c>
       <c r="I65" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -14536,16 +15502,16 @@
         <v>113</v>
       </c>
       <c r="B66" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C66" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D66" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E66" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
       <c r="F66" t="s">
         <v>0</v>
@@ -14557,7 +15523,7 @@
         <v>46</v>
       </c>
       <c r="I66" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -14565,16 +15531,16 @@
         <v>114</v>
       </c>
       <c r="B67" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="C67" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D67" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E67" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="F67" t="s">
         <v>0</v>
@@ -14586,7 +15552,7 @@
         <v>46</v>
       </c>
       <c r="I67" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -14594,16 +15560,16 @@
         <v>115</v>
       </c>
       <c r="B68" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C68" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D68" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E68" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="F68" t="s">
         <v>0</v>
@@ -14615,7 +15581,7 @@
         <v>46</v>
       </c>
       <c r="I68" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -14623,16 +15589,16 @@
         <v>116</v>
       </c>
       <c r="B69" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C69" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D69" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E69" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="F69" t="s">
         <v>0</v>
@@ -14644,7 +15610,7 @@
         <v>46</v>
       </c>
       <c r="I69" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -14652,16 +15618,16 @@
         <v>117</v>
       </c>
       <c r="B70" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="C70" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D70" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E70" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="F70" t="s">
         <v>0</v>
@@ -14673,7 +15639,7 @@
         <v>46</v>
       </c>
       <c r="I70" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -14681,16 +15647,16 @@
         <v>118</v>
       </c>
       <c r="B71" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C71" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="D71" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E71" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="F71" t="s">
         <v>0</v>
@@ -14702,7 +15668,7 @@
         <v>46</v>
       </c>
       <c r="I71" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -14710,16 +15676,16 @@
         <v>119</v>
       </c>
       <c r="B72" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C72" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D72" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="E72" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="F72" t="s">
         <v>0</v>
@@ -14731,7 +15697,7 @@
         <v>46</v>
       </c>
       <c r="I72" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -14739,16 +15705,16 @@
         <v>120</v>
       </c>
       <c r="B73" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C73" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D73" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="E73" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="F73" t="s">
         <v>0</v>
@@ -14760,7 +15726,7 @@
         <v>44</v>
       </c>
       <c r="I73" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -14768,16 +15734,16 @@
         <v>121</v>
       </c>
       <c r="B74" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C74" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D74" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="E74" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="F74" t="s">
         <v>0</v>
@@ -14789,7 +15755,7 @@
         <v>46</v>
       </c>
       <c r="I74" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -14797,16 +15763,16 @@
         <v>122</v>
       </c>
       <c r="B75" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C75" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D75" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E75" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="F75" t="s">
         <v>0</v>
@@ -14818,7 +15784,7 @@
         <v>46</v>
       </c>
       <c r="I75" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -14826,16 +15792,16 @@
         <v>123</v>
       </c>
       <c r="B76" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C76" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D76" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E76" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="F76" t="s">
         <v>0</v>
@@ -14847,7 +15813,7 @@
         <v>46</v>
       </c>
       <c r="I76" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -14855,16 +15821,16 @@
         <v>124</v>
       </c>
       <c r="B77" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C77" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D77" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E77" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="F77" t="s">
         <v>0</v>
@@ -14876,7 +15842,7 @@
         <v>46</v>
       </c>
       <c r="I77" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -14884,16 +15850,16 @@
         <v>125</v>
       </c>
       <c r="B78" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C78" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D78" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E78" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="F78" t="s">
         <v>0</v>
@@ -14905,7 +15871,7 @@
         <v>46</v>
       </c>
       <c r="I78" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -14913,16 +15879,16 @@
         <v>126</v>
       </c>
       <c r="B79" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="C79" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D79" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E79" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
       <c r="F79" t="s">
         <v>0</v>
@@ -14934,7 +15900,7 @@
         <v>47</v>
       </c>
       <c r="I79" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -14942,16 +15908,16 @@
         <v>127</v>
       </c>
       <c r="B80" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C80" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D80" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E80" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="F80" t="s">
         <v>0</v>
@@ -14963,7 +15929,7 @@
         <v>46</v>
       </c>
       <c r="I80" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -14971,16 +15937,16 @@
         <v>128</v>
       </c>
       <c r="B81" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="C81" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D81" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E81" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="F81" t="s">
         <v>0</v>
@@ -14992,7 +15958,7 @@
         <v>46</v>
       </c>
       <c r="I81" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -15000,16 +15966,16 @@
         <v>129</v>
       </c>
       <c r="B82" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="C82" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="D82" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="E82" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="F82" t="s">
         <v>0</v>
@@ -15021,7 +15987,7 @@
         <v>46</v>
       </c>
       <c r="I82" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -15029,28 +15995,619 @@
         <v>130</v>
       </c>
       <c r="B83" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="C83" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
       <c r="D83" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="E83" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="F83" t="s">
         <v>0</v>
       </c>
       <c r="G83" t="s">
+        <v>45</v>
+      </c>
+      <c r="H83">
+        <v>46</v>
+      </c>
+      <c r="I83" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" t="s">
+        <v>131</v>
+      </c>
+      <c r="B84" t="s">
+        <v>228</v>
+      </c>
+      <c r="C84" t="s">
+        <v>244</v>
+      </c>
+      <c r="D84" t="s">
+        <v>261</v>
+      </c>
+      <c r="E84" t="s">
+        <v>326</v>
+      </c>
+      <c r="F84" t="s">
+        <v>28</v>
+      </c>
+      <c r="G84" t="s">
+        <v>43</v>
+      </c>
+      <c r="H84">
+        <v>16</v>
+      </c>
+      <c r="I84" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" t="s">
+        <v>132</v>
+      </c>
+      <c r="B85" t="s">
+        <v>229</v>
+      </c>
+      <c r="C85" t="s">
+        <v>236</v>
+      </c>
+      <c r="D85" t="s">
+        <v>262</v>
+      </c>
+      <c r="E85" t="s">
+        <v>327</v>
+      </c>
+      <c r="F85" t="s">
+        <v>28</v>
+      </c>
+      <c r="G85" t="s">
+        <v>46</v>
+      </c>
+      <c r="H85">
+        <v>19</v>
+      </c>
+      <c r="I85" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86" t="s">
+        <v>133</v>
+      </c>
+      <c r="B86" t="s">
+        <v>230</v>
+      </c>
+      <c r="C86" t="s">
+        <v>236</v>
+      </c>
+      <c r="D86" t="s">
+        <v>262</v>
+      </c>
+      <c r="E86" t="s">
+        <v>328</v>
+      </c>
+      <c r="F86" t="s">
+        <v>28</v>
+      </c>
+      <c r="G86" t="s">
+        <v>46</v>
+      </c>
+      <c r="H86">
+        <v>19</v>
+      </c>
+      <c r="I86" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9">
+      <c r="A87" t="s">
+        <v>134</v>
+      </c>
+      <c r="B87" t="s">
+        <v>231</v>
+      </c>
+      <c r="C87" t="s">
+        <v>236</v>
+      </c>
+      <c r="D87" t="s">
+        <v>263</v>
+      </c>
+      <c r="E87" t="s">
+        <v>314</v>
+      </c>
+      <c r="F87" t="s">
+        <v>0</v>
+      </c>
+      <c r="G87" t="s">
+        <v>45</v>
+      </c>
+      <c r="H87">
+        <v>46</v>
+      </c>
+      <c r="I87" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9">
+      <c r="A88" t="s">
+        <v>135</v>
+      </c>
+      <c r="B88" t="s">
+        <v>232</v>
+      </c>
+      <c r="C88" t="s">
+        <v>236</v>
+      </c>
+      <c r="D88" t="s">
+        <v>263</v>
+      </c>
+      <c r="E88" t="s">
+        <v>314</v>
+      </c>
+      <c r="F88" t="s">
+        <v>0</v>
+      </c>
+      <c r="G88" t="s">
+        <v>45</v>
+      </c>
+      <c r="H88">
+        <v>46</v>
+      </c>
+      <c r="I88" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9">
+      <c r="A89" t="s">
+        <v>136</v>
+      </c>
+      <c r="B89" t="s">
+        <v>233</v>
+      </c>
+      <c r="C89" t="s">
+        <v>244</v>
+      </c>
+      <c r="D89" t="s">
+        <v>263</v>
+      </c>
+      <c r="E89" t="s">
+        <v>314</v>
+      </c>
+      <c r="F89" t="s">
+        <v>0</v>
+      </c>
+      <c r="G89" t="s">
+        <v>45</v>
+      </c>
+      <c r="H89">
+        <v>46</v>
+      </c>
+      <c r="I89" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9">
+      <c r="A90" t="s">
+        <v>137</v>
+      </c>
+      <c r="B90" t="s">
+        <v>234</v>
+      </c>
+      <c r="C90" t="s">
+        <v>240</v>
+      </c>
+      <c r="D90" t="s">
+        <v>264</v>
+      </c>
+      <c r="E90" t="s">
+        <v>329</v>
+      </c>
+      <c r="F90" t="s">
+        <v>0</v>
+      </c>
+      <c r="G90" t="s">
         <v>27</v>
       </c>
-      <c r="H83">
+      <c r="H90">
         <v>28</v>
       </c>
-      <c r="I83" t="s">
-        <v>309</v>
+      <c r="I90" t="s">
+        <v>331</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C1" t="s">
+        <v>333</v>
+      </c>
+      <c r="D1" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2">
+        <v>956.37</v>
+      </c>
+      <c r="C2">
+        <v>742.38</v>
+      </c>
+      <c r="D2">
+        <v>213.99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3">
+        <v>2026</v>
+      </c>
+      <c r="B3">
+        <v>947.26</v>
+      </c>
+      <c r="C3">
+        <v>704.91</v>
+      </c>
+      <c r="D3">
+        <v>242.36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4">
+        <v>2027</v>
+      </c>
+      <c r="B4">
+        <v>1075.78</v>
+      </c>
+      <c r="C4">
+        <v>758.46</v>
+      </c>
+      <c r="D4">
+        <v>317.32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>2028</v>
+      </c>
+      <c r="B5">
+        <v>763.17</v>
+      </c>
+      <c r="C5">
+        <v>443.36</v>
+      </c>
+      <c r="D5">
+        <v>319.81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>2029</v>
+      </c>
+      <c r="B6">
+        <v>915.16</v>
+      </c>
+      <c r="C6">
+        <v>435.61</v>
+      </c>
+      <c r="D6">
+        <v>479.55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>2030</v>
+      </c>
+      <c r="B7">
+        <v>583.89</v>
+      </c>
+      <c r="C7">
+        <v>148.22</v>
+      </c>
+      <c r="D7">
+        <v>435.68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>2031</v>
+      </c>
+      <c r="B8">
+        <v>572.15</v>
+      </c>
+      <c r="C8">
+        <v>143.92</v>
+      </c>
+      <c r="D8">
+        <v>428.23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9">
+        <v>2032</v>
+      </c>
+      <c r="B9">
+        <v>521.7</v>
+      </c>
+      <c r="C9">
+        <v>139.19</v>
+      </c>
+      <c r="D9">
+        <v>382.51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>2033</v>
+      </c>
+      <c r="B10">
+        <v>419.08</v>
+      </c>
+      <c r="C10">
+        <v>129.36</v>
+      </c>
+      <c r="D10">
+        <v>289.71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>2034</v>
+      </c>
+      <c r="B11">
+        <v>645.99</v>
+      </c>
+      <c r="C11">
+        <v>121.9</v>
+      </c>
+      <c r="D11">
+        <v>524.09</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12">
+        <v>2035</v>
+      </c>
+      <c r="B12">
+        <v>640.9400000000001</v>
+      </c>
+      <c r="C12">
+        <v>126.82</v>
+      </c>
+      <c r="D12">
+        <v>514.12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13">
+        <v>2036</v>
+      </c>
+      <c r="B13">
+        <v>586.05</v>
+      </c>
+      <c r="C13">
+        <v>138.24</v>
+      </c>
+      <c r="D13">
+        <v>447.81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14">
+        <v>2037</v>
+      </c>
+      <c r="B14">
+        <v>437.97</v>
+      </c>
+      <c r="C14">
+        <v>175.23</v>
+      </c>
+      <c r="D14">
+        <v>262.74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15">
+        <v>2038</v>
+      </c>
+      <c r="B15">
+        <v>278.04</v>
+      </c>
+      <c r="C15">
+        <v>55.93</v>
+      </c>
+      <c r="D15">
+        <v>222.11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16">
+        <v>2039</v>
+      </c>
+      <c r="B16">
+        <v>269.3</v>
+      </c>
+      <c r="C16">
+        <v>52.51</v>
+      </c>
+      <c r="D16">
+        <v>216.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17">
+        <v>2040</v>
+      </c>
+      <c r="B17">
+        <v>276.5</v>
+      </c>
+      <c r="C17">
+        <v>49.08</v>
+      </c>
+      <c r="D17">
+        <v>227.42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18">
+        <v>2041</v>
+      </c>
+      <c r="B18">
+        <v>223.06</v>
+      </c>
+      <c r="C18">
+        <v>30.65</v>
+      </c>
+      <c r="D18">
+        <v>192.41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19">
+        <v>2042</v>
+      </c>
+      <c r="B19">
+        <v>315.22</v>
+      </c>
+      <c r="C19">
+        <v>29.55</v>
+      </c>
+      <c r="D19">
+        <v>285.67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20">
+        <v>2043</v>
+      </c>
+      <c r="B20">
+        <v>208.1</v>
+      </c>
+      <c r="C20">
+        <v>28.45</v>
+      </c>
+      <c r="D20">
+        <v>179.65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21">
+        <v>2044</v>
+      </c>
+      <c r="B21">
+        <v>203.41</v>
+      </c>
+      <c r="C21">
+        <v>27.35</v>
+      </c>
+      <c r="D21">
+        <v>176.06</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22">
+        <v>2045</v>
+      </c>
+      <c r="B22">
+        <v>196.03</v>
+      </c>
+      <c r="C22">
+        <v>26.25</v>
+      </c>
+      <c r="D22">
+        <v>169.78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23">
+        <v>2046</v>
+      </c>
+      <c r="B23">
+        <v>191.48</v>
+      </c>
+      <c r="C23">
+        <v>25.15</v>
+      </c>
+      <c r="D23">
+        <v>166.33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24">
+        <v>2047</v>
+      </c>
+      <c r="B24">
+        <v>187.32</v>
+      </c>
+      <c r="C24">
+        <v>24.05</v>
+      </c>
+      <c r="D24">
+        <v>163.27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25">
+        <v>2048</v>
+      </c>
+      <c r="B25">
+        <v>170.82</v>
+      </c>
+      <c r="C25">
+        <v>10.85</v>
+      </c>
+      <c r="D25">
+        <v>159.97</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26">
+        <v>2049</v>
+      </c>
+      <c r="B26">
+        <v>168.02</v>
+      </c>
+      <c r="C26">
+        <v>10.85</v>
+      </c>
+      <c r="D26">
+        <v>157.17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27">
+        <v>2050</v>
+      </c>
+      <c r="B27">
+        <v>165.58</v>
+      </c>
+      <c r="C27">
+        <v>10.85</v>
+      </c>
+      <c r="D27">
+        <v>154.73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
History 2026Q3: exports/imports from NBU BOP_m file (API stops at August), September state budget
- loaders/nbu_files: BOP_m.xlsx monthly goods and services (sheet 1.1), shared month-header parser
- history: EXP_USD/IMP_USD/TRADE_BAL fill months the API lacks from the file
- B5_EXTERNAL: 2026Q3 exports/imports are facts once the history has all three months; Q4 keeps the model split
- B6_FISCAL: September 2026 Treasury deficit 99.3 bn UAH (cumulative 669.4 bn)
- refreshed data/history

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UMkgsrK6QTEHqqRgiG741H
</commit_message>
<xml_diff>
--- a/data/history/history.xlsx
+++ b/data/history/history.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1673" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1675" uniqueCount="554">
   <si>
     <t>2015Q1</t>
   </si>
@@ -1309,12 +1309,15 @@
     <t>НБУ API (Госстат); НБУ Wages_m.xlsx; пропуски из MacroStat</t>
   </si>
   <si>
+    <t>НБУ API и BOP_m.xlsx (платёжный баланс)</t>
+  </si>
+  <si>
+    <t>НБУ API (Казначейство)</t>
+  </si>
+  <si>
     <t>НБУ API (платёжный баланс)</t>
   </si>
   <si>
-    <t>НБУ API (Казначейство)</t>
-  </si>
-  <si>
     <t>Минфин (index.minfin.com.ua)</t>
   </si>
   <si>
@@ -1423,10 +1426,10 @@
     <t>Средняя месячная зарплата, среднее за квартал; 2010–2012 из файла НБУ Wages_m; оставшиеся пропуски 2022–2024 из квартальных данных Госстата (лист Salary)</t>
   </si>
   <si>
-    <t>Товары и услуги, кредит, сумма месяцев</t>
-  </si>
-  <si>
-    <t>Товары и услуги, дебет, сумма месяцев</t>
+    <t>Товары и услуги, кредит, сумма месяцев; последние месяцы до API из файла BOP_m</t>
+  </si>
+  <si>
+    <t>Товары и услуги, дебет, сумма месяцев; последние месяцы до API из файла BOP_m</t>
   </si>
   <si>
     <t>EXP_USD − IMP_USD</t>
@@ -1667,6 +1670,12 @@
   </si>
   <si>
     <t>external</t>
+  </si>
+  <si>
+    <t>external_interest</t>
+  </si>
+  <si>
+    <t>external_repayment</t>
   </si>
   <si>
     <t>year</t>
@@ -3156,6 +3165,9 @@
       <c r="AU8">
         <v>39.1</v>
       </c>
+      <c r="AV8">
+        <v>38.4</v>
+      </c>
     </row>
     <row r="9" spans="1:49">
       <c r="A9" t="s">
@@ -3303,7 +3315,7 @@
         <v>44.69044673913044</v>
       </c>
       <c r="AW9">
-        <v>44.9262125</v>
+        <v>45.02476</v>
       </c>
     </row>
     <row r="10" spans="1:49">
@@ -3452,7 +3464,7 @@
         <v>44.8624</v>
       </c>
       <c r="AW10">
-        <v>45.051</v>
+        <v>45.5293</v>
       </c>
     </row>
     <row r="11" spans="1:49">
@@ -3601,7 +3613,7 @@
         <v>16</v>
       </c>
       <c r="AW11">
-        <v>16</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="12" spans="1:49">
@@ -3746,6 +3758,9 @@
       <c r="AU12">
         <v>19.83115822623704</v>
       </c>
+      <c r="AV12">
+        <v>19.98829703300498</v>
+      </c>
     </row>
     <row r="13" spans="1:49">
       <c r="A13" t="s">
@@ -3889,6 +3904,9 @@
       <c r="AU13">
         <v>10.05497450613516</v>
       </c>
+      <c r="AV13">
+        <v>10.42740907713206</v>
+      </c>
     </row>
     <row r="14" spans="1:49">
       <c r="A14" t="s">
@@ -4347,6 +4365,9 @@
       <c r="AU17">
         <v>31419.66666666667</v>
       </c>
+      <c r="AV17">
+        <v>32429.33333333333</v>
+      </c>
     </row>
     <row r="18" spans="1:48">
       <c r="A18" t="s">
@@ -4490,6 +4511,9 @@
       <c r="AU18">
         <v>14387</v>
       </c>
+      <c r="AV18">
+        <v>12187</v>
+      </c>
     </row>
     <row r="19" spans="1:48">
       <c r="A19" t="s">
@@ -4633,6 +4657,9 @@
       <c r="AU19">
         <v>31814</v>
       </c>
+      <c r="AV19">
+        <v>32342</v>
+      </c>
     </row>
     <row r="20" spans="1:48">
       <c r="A20" t="s">
@@ -4775,6 +4802,9 @@
       </c>
       <c r="AU20">
         <v>-17427</v>
+      </c>
+      <c r="AV20">
+        <v>-20155</v>
       </c>
     </row>
     <row r="21" spans="1:48">
@@ -10995,6 +11025,9 @@
       <c r="AU36">
         <v>9.133333333333335</v>
       </c>
+      <c r="AV36">
+        <v>6.199999999999998</v>
+      </c>
     </row>
     <row r="37" spans="1:48">
       <c r="A37" t="s">
@@ -11281,6 +11314,9 @@
       <c r="AU38">
         <v>914723.0858999999</v>
       </c>
+      <c r="AV38">
+        <v>917327.197</v>
+      </c>
     </row>
     <row r="39" spans="1:48">
       <c r="A39" t="s">
@@ -11424,6 +11460,9 @@
       <c r="AU39">
         <v>4139259.1604</v>
       </c>
+      <c r="AV39">
+        <v>4195653.3797</v>
+      </c>
     </row>
     <row r="40" spans="1:48">
       <c r="A40" t="s">
@@ -11567,6 +11606,9 @@
       <c r="AU40">
         <v>15.55165556739514</v>
       </c>
+      <c r="AV40">
+        <v>17.75376782523249</v>
+      </c>
     </row>
     <row r="41" spans="1:48">
       <c r="A41" t="s">
@@ -11710,6 +11752,9 @@
       <c r="AU41">
         <v>29.2948390853322</v>
       </c>
+      <c r="AV41">
+        <v>29.08101818194272</v>
+      </c>
     </row>
     <row r="42" spans="1:48">
       <c r="A42" t="s">
@@ -11853,6 +11898,9 @@
       <c r="AU42">
         <v>10.38844073943397</v>
       </c>
+      <c r="AV42">
+        <v>10.31664473658278</v>
+      </c>
     </row>
     <row r="43" spans="1:48">
       <c r="A43" t="s">
@@ -13423,6 +13471,9 @@
       <c r="AU53">
         <v>9490799.6</v>
       </c>
+      <c r="AV53">
+        <v>9538348.800000001</v>
+      </c>
     </row>
     <row r="54" spans="1:48">
       <c r="A54" t="s">
@@ -14291,6 +14342,9 @@
       <c r="AU61">
         <v>5466.566666666667</v>
       </c>
+      <c r="AV61">
+        <v>5493.233333333334</v>
+      </c>
     </row>
     <row r="62" spans="1:48">
       <c r="A62" t="s">
@@ -16239,6 +16293,9 @@
       <c r="AU75">
         <v>14.7</v>
       </c>
+      <c r="AV75">
+        <v>13.6</v>
+      </c>
     </row>
     <row r="76" spans="1:48">
       <c r="A76" t="s">
@@ -16382,6 +16439,9 @@
       <c r="AU76">
         <v>9.9</v>
       </c>
+      <c r="AV76">
+        <v>3.4</v>
+      </c>
     </row>
     <row r="77" spans="1:48">
       <c r="A77" t="s">
@@ -17865,6 +17925,9 @@
       <c r="AU87">
         <v>6237.14266107</v>
       </c>
+      <c r="AV87">
+        <v>4467.46851447</v>
+      </c>
     </row>
     <row r="88" spans="1:48">
       <c r="A88" t="s">
@@ -18008,6 +18071,9 @@
       <c r="AU88">
         <v>2178.587996930001</v>
       </c>
+      <c r="AV88">
+        <v>1933.66236314</v>
+      </c>
     </row>
     <row r="89" spans="1:48">
       <c r="A89" t="s">
@@ -18151,6 +18217,9 @@
       <c r="AU89">
         <v>682.17082755</v>
       </c>
+      <c r="AV89">
+        <v>649.24482759</v>
+      </c>
     </row>
     <row r="90" spans="1:48">
       <c r="A90" t="s">
@@ -18294,6 +18363,9 @@
       <c r="AU90">
         <v>3323.99618793</v>
       </c>
+      <c r="AV90">
+        <v>3387.55877592</v>
+      </c>
     </row>
     <row r="91" spans="1:48">
       <c r="A91" t="s">
@@ -18437,6 +18509,9 @@
       <c r="AU91">
         <v>437.7822446900002</v>
       </c>
+      <c r="AV91">
+        <v>411.3390702800002</v>
+      </c>
     </row>
     <row r="92" spans="1:48">
       <c r="A92" t="s">
@@ -18580,6 +18655,9 @@
       <c r="AU92">
         <v>3451.173779139996</v>
       </c>
+      <c r="AV92">
+        <v>3109.25742917</v>
+      </c>
     </row>
     <row r="93" spans="1:48">
       <c r="A93" t="s">
@@ -18723,6 +18801,9 @@
       <c r="AU93">
         <v>533.57196893</v>
       </c>
+      <c r="AV93">
+        <v>509.52608051</v>
+      </c>
     </row>
     <row r="94" spans="1:48">
       <c r="A94" t="s">
@@ -18866,6 +18947,9 @@
       <c r="AU94">
         <v>339.2838354299998</v>
       </c>
+      <c r="AV94">
+        <v>311.4197745599998</v>
+      </c>
     </row>
     <row r="95" spans="1:48">
       <c r="A95" t="s">
@@ -19009,6 +19093,9 @@
       <c r="AU95">
         <v>196.9822311900001</v>
       </c>
+      <c r="AV95">
+        <v>188.10629171</v>
+      </c>
     </row>
     <row r="96" spans="1:48">
       <c r="A96" t="s">
@@ -19152,8 +19239,11 @@
       <c r="AU96">
         <v>966.9308393500008</v>
       </c>
-    </row>
-    <row r="97" spans="1:47">
+      <c r="AV96">
+        <v>1203.50340813</v>
+      </c>
+    </row>
+    <row r="97" spans="1:48">
       <c r="A97" t="s">
         <v>173</v>
       </c>
@@ -19295,8 +19385,11 @@
       <c r="AU97">
         <v>1227.76045312</v>
       </c>
-    </row>
-    <row r="98" spans="1:47">
+      <c r="AV97">
+        <v>714.61069847</v>
+      </c>
+    </row>
+    <row r="98" spans="1:48">
       <c r="A98" t="s">
         <v>174</v>
       </c>
@@ -19438,8 +19531,11 @@
       <c r="AU98">
         <v>1256.43277541</v>
       </c>
-    </row>
-    <row r="99" spans="1:47">
+      <c r="AV98">
+        <v>1208.091834829999</v>
+      </c>
+    </row>
+    <row r="99" spans="1:48">
       <c r="A99" t="s">
         <v>175</v>
       </c>
@@ -19581,8 +19677,11 @@
       <c r="AU99">
         <v>440.674090939998</v>
       </c>
-    </row>
-    <row r="100" spans="1:47">
+      <c r="AV99">
+        <v>413.133863630001</v>
+      </c>
+    </row>
+    <row r="100" spans="1:48">
       <c r="A100" t="s">
         <v>176</v>
       </c>
@@ -19724,8 +19823,11 @@
       <c r="AU100">
         <v>11435.77814950999</v>
       </c>
-    </row>
-    <row r="101" spans="1:47">
+      <c r="AV100">
+        <v>12807.93434983</v>
+      </c>
+    </row>
+    <row r="101" spans="1:48">
       <c r="A101" t="s">
         <v>177</v>
       </c>
@@ -19867,8 +19969,11 @@
       <c r="AU101">
         <v>435.9155225100026</v>
       </c>
-    </row>
-    <row r="102" spans="1:47">
+      <c r="AV101">
+        <v>602.5706533399989</v>
+      </c>
+    </row>
+    <row r="102" spans="1:48">
       <c r="A102" t="s">
         <v>178</v>
       </c>
@@ -20010,8 +20115,11 @@
       <c r="AU102">
         <v>2701.816436300007</v>
       </c>
-    </row>
-    <row r="103" spans="1:47">
+      <c r="AV102">
+        <v>1759.572064420003</v>
+      </c>
+    </row>
+    <row r="103" spans="1:48">
       <c r="A103" t="s">
         <v>179</v>
       </c>
@@ -20139,7 +20247,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="104" spans="1:47">
+    <row r="104" spans="1:48">
       <c r="A104" t="s">
         <v>180</v>
       </c>
@@ -20264,7 +20372,7 @@
         <v>243.6666666666667</v>
       </c>
     </row>
-    <row r="105" spans="1:47">
+    <row r="105" spans="1:48">
       <c r="A105" t="s">
         <v>181</v>
       </c>
@@ -20404,7 +20512,7 @@
         <v>1323.333333333333</v>
       </c>
     </row>
-    <row r="106" spans="1:47">
+    <row r="106" spans="1:48">
       <c r="A106" t="s">
         <v>182</v>
       </c>
@@ -20544,7 +20652,7 @@
         <v>463.3333333333333</v>
       </c>
     </row>
-    <row r="107" spans="1:47">
+    <row r="107" spans="1:48">
       <c r="A107" t="s">
         <v>183</v>
       </c>
@@ -20687,7 +20795,7 @@
         <v>1653117.9</v>
       </c>
     </row>
-    <row r="108" spans="1:47">
+    <row r="108" spans="1:48">
       <c r="A108" t="s">
         <v>184</v>
       </c>
@@ -20830,7 +20938,7 @@
         <v>237170.3</v>
       </c>
     </row>
-    <row r="109" spans="1:47">
+    <row r="109" spans="1:48">
       <c r="A109" t="s">
         <v>185</v>
       </c>
@@ -20973,7 +21081,7 @@
         <v>88222.2</v>
       </c>
     </row>
-    <row r="110" spans="1:47">
+    <row r="110" spans="1:48">
       <c r="A110" t="s">
         <v>186</v>
       </c>
@@ -21116,7 +21224,7 @@
         <v>78150.99999999999</v>
       </c>
     </row>
-    <row r="111" spans="1:47">
+    <row r="111" spans="1:48">
       <c r="A111" t="s">
         <v>187</v>
       </c>
@@ -21259,7 +21367,7 @@
         <v>170583</v>
       </c>
     </row>
-    <row r="112" spans="1:47">
+    <row r="112" spans="1:48">
       <c r="A112" t="s">
         <v>188</v>
       </c>
@@ -25651,7 +25759,7 @@
         <v>422</v>
       </c>
       <c r="E2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F2" t="s">
         <v>0</v>
@@ -25663,7 +25771,7 @@
         <v>46</v>
       </c>
       <c r="I2" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -25680,7 +25788,7 @@
         <v>422</v>
       </c>
       <c r="E3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F3" t="s">
         <v>0</v>
@@ -25692,7 +25800,7 @@
         <v>46</v>
       </c>
       <c r="I3" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -25709,7 +25817,7 @@
         <v>422</v>
       </c>
       <c r="E4" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F4" t="s">
         <v>0</v>
@@ -25721,7 +25829,7 @@
         <v>46</v>
       </c>
       <c r="I4" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -25738,7 +25846,7 @@
         <v>422</v>
       </c>
       <c r="E5" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
@@ -25750,7 +25858,7 @@
         <v>46</v>
       </c>
       <c r="I5" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -25767,7 +25875,7 @@
         <v>423</v>
       </c>
       <c r="E6" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F6" t="s">
         <v>0</v>
@@ -25779,7 +25887,7 @@
         <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -25796,7 +25904,7 @@
         <v>422</v>
       </c>
       <c r="E7" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F7" t="s">
         <v>0</v>
@@ -25808,7 +25916,7 @@
         <v>47</v>
       </c>
       <c r="I7" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -25825,19 +25933,19 @@
         <v>424</v>
       </c>
       <c r="E8" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F8" t="s">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H8">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I8" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -25854,7 +25962,7 @@
         <v>425</v>
       </c>
       <c r="E9" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F9" t="s">
         <v>0</v>
@@ -25866,7 +25974,7 @@
         <v>48</v>
       </c>
       <c r="I9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -25883,7 +25991,7 @@
         <v>425</v>
       </c>
       <c r="E10" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F10" t="s">
         <v>0</v>
@@ -25895,7 +26003,7 @@
         <v>48</v>
       </c>
       <c r="I10" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -25912,7 +26020,7 @@
         <v>426</v>
       </c>
       <c r="E11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F11" t="s">
         <v>0</v>
@@ -25924,7 +26032,7 @@
         <v>48</v>
       </c>
       <c r="I11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -25941,19 +26049,19 @@
         <v>426</v>
       </c>
       <c r="E12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F12" t="s">
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H12">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -25970,19 +26078,19 @@
         <v>426</v>
       </c>
       <c r="E13" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F13" t="s">
         <v>0</v>
       </c>
       <c r="G13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H13">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I13" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -25999,7 +26107,7 @@
         <v>427</v>
       </c>
       <c r="E14" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F14" t="s">
         <v>0</v>
@@ -26011,7 +26119,7 @@
         <v>44</v>
       </c>
       <c r="I14" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -26028,7 +26136,7 @@
         <v>428</v>
       </c>
       <c r="E15" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F15" t="s">
         <v>0</v>
@@ -26040,7 +26148,7 @@
         <v>28</v>
       </c>
       <c r="I15" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -26057,7 +26165,7 @@
         <v>428</v>
       </c>
       <c r="E16" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F16" t="s">
         <v>0</v>
@@ -26069,7 +26177,7 @@
         <v>28</v>
       </c>
       <c r="I16" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -26086,19 +26194,19 @@
         <v>429</v>
       </c>
       <c r="E17" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F17" t="s">
         <v>0</v>
       </c>
       <c r="G17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H17">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I17" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -26115,19 +26223,19 @@
         <v>430</v>
       </c>
       <c r="E18" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F18" t="s">
         <v>0</v>
       </c>
       <c r="G18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H18">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I18" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -26144,19 +26252,19 @@
         <v>430</v>
       </c>
       <c r="E19" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F19" t="s">
         <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H19">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I19" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -26173,19 +26281,19 @@
         <v>423</v>
       </c>
       <c r="E20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F20" t="s">
         <v>0</v>
       </c>
       <c r="G20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H20">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I20" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -26202,7 +26310,7 @@
         <v>426</v>
       </c>
       <c r="E21" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F21" t="s">
         <v>0</v>
@@ -26214,7 +26322,7 @@
         <v>47</v>
       </c>
       <c r="I21" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -26231,7 +26339,7 @@
         <v>422</v>
       </c>
       <c r="E22" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F22" t="s">
         <v>0</v>
@@ -26243,7 +26351,7 @@
         <v>46</v>
       </c>
       <c r="I22" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -26260,7 +26368,7 @@
         <v>427</v>
       </c>
       <c r="E23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F23" t="s">
         <v>0</v>
@@ -26272,7 +26380,7 @@
         <v>28</v>
       </c>
       <c r="I23" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -26289,7 +26397,7 @@
         <v>431</v>
       </c>
       <c r="E24" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F24" t="s">
         <v>0</v>
@@ -26301,7 +26409,7 @@
         <v>46</v>
       </c>
       <c r="I24" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -26318,13 +26426,13 @@
         <v>423</v>
       </c>
       <c r="E25" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="I25" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -26338,10 +26446,10 @@
         <v>414</v>
       </c>
       <c r="D26" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E26" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F26" t="s">
         <v>0</v>
@@ -26353,7 +26461,7 @@
         <v>46</v>
       </c>
       <c r="I26" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -26370,13 +26478,13 @@
         <v>423</v>
       </c>
       <c r="E27" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="H27">
         <v>0</v>
       </c>
       <c r="I27" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -26390,10 +26498,10 @@
         <v>415</v>
       </c>
       <c r="D28" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E28" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F28" t="s">
         <v>0</v>
@@ -26405,7 +26513,7 @@
         <v>46</v>
       </c>
       <c r="I28" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -26422,7 +26530,7 @@
         <v>427</v>
       </c>
       <c r="E29" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F29" t="s">
         <v>0</v>
@@ -26434,7 +26542,7 @@
         <v>40</v>
       </c>
       <c r="I29" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -26448,10 +26556,10 @@
         <v>417</v>
       </c>
       <c r="D30" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E30" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F30" t="s">
         <v>12</v>
@@ -26463,7 +26571,7 @@
         <v>34</v>
       </c>
       <c r="I30" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -26480,7 +26588,7 @@
         <v>422</v>
       </c>
       <c r="E31" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F31" t="s">
         <v>0</v>
@@ -26492,7 +26600,7 @@
         <v>46</v>
       </c>
       <c r="I31" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -26509,7 +26617,7 @@
         <v>422</v>
       </c>
       <c r="E32" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F32" t="s">
         <v>0</v>
@@ -26521,7 +26629,7 @@
         <v>46</v>
       </c>
       <c r="I32" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -26538,7 +26646,7 @@
         <v>422</v>
       </c>
       <c r="E33" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F33" t="s">
         <v>0</v>
@@ -26550,7 +26658,7 @@
         <v>46</v>
       </c>
       <c r="I33" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -26567,7 +26675,7 @@
         <v>422</v>
       </c>
       <c r="E34" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F34" t="s">
         <v>0</v>
@@ -26579,7 +26687,7 @@
         <v>46</v>
       </c>
       <c r="I34" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -26596,7 +26704,7 @@
         <v>422</v>
       </c>
       <c r="E35" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F35" t="s">
         <v>0</v>
@@ -26608,7 +26716,7 @@
         <v>46</v>
       </c>
       <c r="I35" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -26625,7 +26733,7 @@
         <v>422</v>
       </c>
       <c r="E36" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F36" t="s">
         <v>0</v>
@@ -26637,7 +26745,7 @@
         <v>46</v>
       </c>
       <c r="I36" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -26654,7 +26762,7 @@
         <v>422</v>
       </c>
       <c r="E37" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F37" t="s">
         <v>0</v>
@@ -26666,7 +26774,7 @@
         <v>46</v>
       </c>
       <c r="I37" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -26683,7 +26791,7 @@
         <v>422</v>
       </c>
       <c r="E38" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F38" t="s">
         <v>0</v>
@@ -26695,7 +26803,7 @@
         <v>46</v>
       </c>
       <c r="I38" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -26712,7 +26820,7 @@
         <v>422</v>
       </c>
       <c r="E39" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F39" t="s">
         <v>0</v>
@@ -26724,7 +26832,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -26741,7 +26849,7 @@
         <v>422</v>
       </c>
       <c r="E40" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F40" t="s">
         <v>0</v>
@@ -26753,7 +26861,7 @@
         <v>46</v>
       </c>
       <c r="I40" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -26770,7 +26878,7 @@
         <v>422</v>
       </c>
       <c r="E41" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F41" t="s">
         <v>0</v>
@@ -26782,7 +26890,7 @@
         <v>46</v>
       </c>
       <c r="I41" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -26799,7 +26907,7 @@
         <v>422</v>
       </c>
       <c r="E42" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F42" t="s">
         <v>0</v>
@@ -26811,7 +26919,7 @@
         <v>46</v>
       </c>
       <c r="I42" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -26828,7 +26936,7 @@
         <v>422</v>
       </c>
       <c r="E43" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F43" t="s">
         <v>0</v>
@@ -26840,7 +26948,7 @@
         <v>46</v>
       </c>
       <c r="I43" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -26857,7 +26965,7 @@
         <v>422</v>
       </c>
       <c r="E44" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F44" t="s">
         <v>0</v>
@@ -26869,7 +26977,7 @@
         <v>46</v>
       </c>
       <c r="I44" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -26886,7 +26994,7 @@
         <v>422</v>
       </c>
       <c r="E45" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F45" t="s">
         <v>0</v>
@@ -26898,7 +27006,7 @@
         <v>46</v>
       </c>
       <c r="I45" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -26915,7 +27023,7 @@
         <v>422</v>
       </c>
       <c r="E46" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F46" t="s">
         <v>0</v>
@@ -26927,7 +27035,7 @@
         <v>46</v>
       </c>
       <c r="I46" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -26944,7 +27052,7 @@
         <v>422</v>
       </c>
       <c r="E47" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F47" t="s">
         <v>0</v>
@@ -26956,7 +27064,7 @@
         <v>46</v>
       </c>
       <c r="I47" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -26973,7 +27081,7 @@
         <v>422</v>
       </c>
       <c r="E48" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F48" t="s">
         <v>0</v>
@@ -26985,7 +27093,7 @@
         <v>46</v>
       </c>
       <c r="I48" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -27002,7 +27110,7 @@
         <v>422</v>
       </c>
       <c r="E49" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F49" t="s">
         <v>0</v>
@@ -27014,7 +27122,7 @@
         <v>46</v>
       </c>
       <c r="I49" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -27031,7 +27139,7 @@
         <v>422</v>
       </c>
       <c r="E50" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F50" t="s">
         <v>0</v>
@@ -27043,7 +27151,7 @@
         <v>46</v>
       </c>
       <c r="I50" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -27060,7 +27168,7 @@
         <v>422</v>
       </c>
       <c r="E51" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F51" t="s">
         <v>0</v>
@@ -27072,7 +27180,7 @@
         <v>46</v>
       </c>
       <c r="I51" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -27089,7 +27197,7 @@
         <v>422</v>
       </c>
       <c r="E52" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F52" t="s">
         <v>0</v>
@@ -27101,7 +27209,7 @@
         <v>46</v>
       </c>
       <c r="I52" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -27118,7 +27226,7 @@
         <v>422</v>
       </c>
       <c r="E53" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F53" t="s">
         <v>0</v>
@@ -27130,7 +27238,7 @@
         <v>46</v>
       </c>
       <c r="I53" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -27147,7 +27255,7 @@
         <v>422</v>
       </c>
       <c r="E54" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F54" t="s">
         <v>0</v>
@@ -27159,7 +27267,7 @@
         <v>46</v>
       </c>
       <c r="I54" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -27176,7 +27284,7 @@
         <v>422</v>
       </c>
       <c r="E55" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F55" t="s">
         <v>0</v>
@@ -27188,7 +27296,7 @@
         <v>46</v>
       </c>
       <c r="I55" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -27205,7 +27313,7 @@
         <v>422</v>
       </c>
       <c r="E56" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F56" t="s">
         <v>0</v>
@@ -27217,7 +27325,7 @@
         <v>46</v>
       </c>
       <c r="I56" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -27234,7 +27342,7 @@
         <v>422</v>
       </c>
       <c r="E57" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F57" t="s">
         <v>0</v>
@@ -27246,7 +27354,7 @@
         <v>46</v>
       </c>
       <c r="I57" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -27263,7 +27371,7 @@
         <v>422</v>
       </c>
       <c r="E58" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F58" t="s">
         <v>0</v>
@@ -27275,7 +27383,7 @@
         <v>46</v>
       </c>
       <c r="I58" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -27292,7 +27400,7 @@
         <v>422</v>
       </c>
       <c r="E59" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F59" t="s">
         <v>0</v>
@@ -27304,7 +27412,7 @@
         <v>46</v>
       </c>
       <c r="I59" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -27321,7 +27429,7 @@
         <v>422</v>
       </c>
       <c r="E60" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F60" t="s">
         <v>0</v>
@@ -27333,7 +27441,7 @@
         <v>46</v>
       </c>
       <c r="I60" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -27350,7 +27458,7 @@
         <v>422</v>
       </c>
       <c r="E61" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F61" t="s">
         <v>0</v>
@@ -27362,7 +27470,7 @@
         <v>46</v>
       </c>
       <c r="I61" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -27379,7 +27487,7 @@
         <v>422</v>
       </c>
       <c r="E62" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F62" t="s">
         <v>0</v>
@@ -27391,7 +27499,7 @@
         <v>47</v>
       </c>
       <c r="I62" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -27405,10 +27513,10 @@
         <v>418</v>
       </c>
       <c r="D63" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E63" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F63" t="s">
         <v>0</v>
@@ -27420,7 +27528,7 @@
         <v>47</v>
       </c>
       <c r="I63" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -27434,10 +27542,10 @@
         <v>418</v>
       </c>
       <c r="D64" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E64" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F64" t="s">
         <v>0</v>
@@ -27449,7 +27557,7 @@
         <v>46</v>
       </c>
       <c r="I64" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -27466,19 +27574,19 @@
         <v>422</v>
       </c>
       <c r="E65" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F65" t="s">
         <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H65">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I65" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -27495,7 +27603,7 @@
         <v>422</v>
       </c>
       <c r="E66" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F66" t="s">
         <v>0</v>
@@ -27507,7 +27615,7 @@
         <v>46</v>
       </c>
       <c r="I66" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -27524,19 +27632,19 @@
         <v>426</v>
       </c>
       <c r="E67" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F67" t="s">
         <v>0</v>
       </c>
       <c r="G67" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H67">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I67" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -27553,19 +27661,19 @@
         <v>426</v>
       </c>
       <c r="E68" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F68" t="s">
         <v>0</v>
       </c>
       <c r="G68" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H68">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I68" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -27582,19 +27690,19 @@
         <v>426</v>
       </c>
       <c r="E69" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F69" t="s">
         <v>0</v>
       </c>
       <c r="G69" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H69">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I69" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -27611,19 +27719,19 @@
         <v>426</v>
       </c>
       <c r="E70" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F70" t="s">
         <v>0</v>
       </c>
       <c r="G70" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H70">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I70" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -27640,19 +27748,19 @@
         <v>426</v>
       </c>
       <c r="E71" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F71" t="s">
         <v>0</v>
       </c>
       <c r="G71" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H71">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I71" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -27669,7 +27777,7 @@
         <v>431</v>
       </c>
       <c r="E72" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F72" t="s">
         <v>0</v>
@@ -27681,7 +27789,7 @@
         <v>46</v>
       </c>
       <c r="I72" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -27698,7 +27806,7 @@
         <v>431</v>
       </c>
       <c r="E73" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F73" t="s">
         <v>0</v>
@@ -27710,7 +27818,7 @@
         <v>44</v>
       </c>
       <c r="I73" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -27727,7 +27835,7 @@
         <v>431</v>
       </c>
       <c r="E74" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F74" t="s">
         <v>0</v>
@@ -27739,7 +27847,7 @@
         <v>46</v>
       </c>
       <c r="I74" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -27753,10 +27861,10 @@
         <v>414</v>
       </c>
       <c r="D75" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E75" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F75" t="s">
         <v>0</v>
@@ -27768,7 +27876,7 @@
         <v>46</v>
       </c>
       <c r="I75" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -27782,10 +27890,10 @@
         <v>414</v>
       </c>
       <c r="D76" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E76" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F76" t="s">
         <v>0</v>
@@ -27797,7 +27905,7 @@
         <v>46</v>
       </c>
       <c r="I76" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -27811,10 +27919,10 @@
         <v>414</v>
       </c>
       <c r="D77" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E77" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F77" t="s">
         <v>0</v>
@@ -27826,7 +27934,7 @@
         <v>46</v>
       </c>
       <c r="I77" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -27840,10 +27948,10 @@
         <v>414</v>
       </c>
       <c r="D78" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E78" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F78" t="s">
         <v>0</v>
@@ -27855,7 +27963,7 @@
         <v>46</v>
       </c>
       <c r="I78" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -27872,7 +27980,7 @@
         <v>426</v>
       </c>
       <c r="E79" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F79" t="s">
         <v>0</v>
@@ -27884,7 +27992,7 @@
         <v>47</v>
       </c>
       <c r="I79" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -27901,7 +28009,7 @@
         <v>426</v>
       </c>
       <c r="E80" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F80" t="s">
         <v>0</v>
@@ -27913,7 +28021,7 @@
         <v>46</v>
       </c>
       <c r="I80" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -27930,7 +28038,7 @@
         <v>426</v>
       </c>
       <c r="E81" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F81" t="s">
         <v>0</v>
@@ -27942,7 +28050,7 @@
         <v>46</v>
       </c>
       <c r="I81" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -27956,22 +28064,22 @@
         <v>406</v>
       </c>
       <c r="D82" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E82" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F82" t="s">
         <v>0</v>
       </c>
       <c r="G82" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H82">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I82" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -27985,10 +28093,10 @@
         <v>412</v>
       </c>
       <c r="D83" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E83" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F83" t="s">
         <v>0</v>
@@ -28000,7 +28108,7 @@
         <v>46</v>
       </c>
       <c r="I83" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -28014,10 +28122,10 @@
         <v>414</v>
       </c>
       <c r="D84" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E84" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F84" t="s">
         <v>28</v>
@@ -28029,7 +28137,7 @@
         <v>16</v>
       </c>
       <c r="I84" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -28043,10 +28151,10 @@
         <v>406</v>
       </c>
       <c r="D85" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E85" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F85" t="s">
         <v>28</v>
@@ -28058,7 +28166,7 @@
         <v>19</v>
       </c>
       <c r="I85" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="86" spans="1:9">
@@ -28072,10 +28180,10 @@
         <v>406</v>
       </c>
       <c r="D86" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E86" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F86" t="s">
         <v>28</v>
@@ -28087,7 +28195,7 @@
         <v>19</v>
       </c>
       <c r="I86" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -28101,10 +28209,10 @@
         <v>406</v>
       </c>
       <c r="D87" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E87" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F87" t="s">
         <v>0</v>
@@ -28116,7 +28224,7 @@
         <v>46</v>
       </c>
       <c r="I87" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -28130,10 +28238,10 @@
         <v>406</v>
       </c>
       <c r="D88" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E88" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F88" t="s">
         <v>0</v>
@@ -28145,7 +28253,7 @@
         <v>46</v>
       </c>
       <c r="I88" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -28159,10 +28267,10 @@
         <v>414</v>
       </c>
       <c r="D89" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E89" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F89" t="s">
         <v>0</v>
@@ -28174,7 +28282,7 @@
         <v>46</v>
       </c>
       <c r="I89" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -28188,22 +28296,22 @@
         <v>412</v>
       </c>
       <c r="D90" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="E90" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F90" t="s">
         <v>0</v>
       </c>
       <c r="G90" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H90">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I90" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -28217,10 +28325,10 @@
         <v>410</v>
       </c>
       <c r="D91" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E91" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F91" t="s">
         <v>0</v>
@@ -28232,7 +28340,7 @@
         <v>28</v>
       </c>
       <c r="I91" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -28249,7 +28357,7 @@
         <v>422</v>
       </c>
       <c r="E92" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F92" t="s">
         <v>0</v>
@@ -28261,7 +28369,7 @@
         <v>46</v>
       </c>
       <c r="I92" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -28278,7 +28386,7 @@
         <v>422</v>
       </c>
       <c r="E93" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F93" t="s">
         <v>0</v>
@@ -28290,7 +28398,7 @@
         <v>46</v>
       </c>
       <c r="I93" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -28307,7 +28415,7 @@
         <v>422</v>
       </c>
       <c r="E94" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F94" t="s">
         <v>0</v>
@@ -28319,7 +28427,7 @@
         <v>46</v>
       </c>
       <c r="I94" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -28336,7 +28444,7 @@
         <v>422</v>
       </c>
       <c r="E95" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F95" t="s">
         <v>0</v>
@@ -28348,7 +28456,7 @@
         <v>46</v>
       </c>
       <c r="I95" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -28365,7 +28473,7 @@
         <v>422</v>
       </c>
       <c r="E96" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F96" t="s">
         <v>0</v>
@@ -28377,7 +28485,7 @@
         <v>46</v>
       </c>
       <c r="I96" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -28394,7 +28502,7 @@
         <v>422</v>
       </c>
       <c r="E97" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F97" t="s">
         <v>0</v>
@@ -28406,7 +28514,7 @@
         <v>46</v>
       </c>
       <c r="I97" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -28423,7 +28531,7 @@
         <v>422</v>
       </c>
       <c r="E98" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F98" t="s">
         <v>0</v>
@@ -28435,7 +28543,7 @@
         <v>46</v>
       </c>
       <c r="I98" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -28452,7 +28560,7 @@
         <v>422</v>
       </c>
       <c r="E99" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F99" t="s">
         <v>0</v>
@@ -28464,7 +28572,7 @@
         <v>46</v>
       </c>
       <c r="I99" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="100" spans="1:9">
@@ -28481,7 +28589,7 @@
         <v>422</v>
       </c>
       <c r="E100" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="F100" t="s">
         <v>0</v>
@@ -28493,7 +28601,7 @@
         <v>46</v>
       </c>
       <c r="I100" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -28510,7 +28618,7 @@
         <v>422</v>
       </c>
       <c r="E101" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F101" t="s">
         <v>0</v>
@@ -28522,7 +28630,7 @@
         <v>46</v>
       </c>
       <c r="I101" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -28539,7 +28647,7 @@
         <v>422</v>
       </c>
       <c r="E102" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F102" t="s">
         <v>0</v>
@@ -28551,7 +28659,7 @@
         <v>46</v>
       </c>
       <c r="I102" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="103" spans="1:9">
@@ -28568,7 +28676,7 @@
         <v>422</v>
       </c>
       <c r="E103" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F103" t="s">
         <v>0</v>
@@ -28580,7 +28688,7 @@
         <v>46</v>
       </c>
       <c r="I103" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -28594,22 +28702,22 @@
         <v>418</v>
       </c>
       <c r="D104" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E104" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F104" t="s">
         <v>0</v>
       </c>
       <c r="G104" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H104">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I104" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -28623,22 +28731,22 @@
         <v>418</v>
       </c>
       <c r="D105" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E105" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F105" t="s">
         <v>0</v>
       </c>
       <c r="G105" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H105">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I105" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -28655,7 +28763,7 @@
         <v>422</v>
       </c>
       <c r="E106" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F106" t="s">
         <v>0</v>
@@ -28667,7 +28775,7 @@
         <v>47</v>
       </c>
       <c r="I106" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -28684,7 +28792,7 @@
         <v>422</v>
       </c>
       <c r="E107" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="F107" t="s">
         <v>0</v>
@@ -28696,7 +28804,7 @@
         <v>47</v>
       </c>
       <c r="I107" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -28713,7 +28821,7 @@
         <v>422</v>
       </c>
       <c r="E108" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F108" t="s">
         <v>0</v>
@@ -28725,7 +28833,7 @@
         <v>47</v>
       </c>
       <c r="I108" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -28742,7 +28850,7 @@
         <v>422</v>
       </c>
       <c r="E109" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F109" t="s">
         <v>0</v>
@@ -28754,7 +28862,7 @@
         <v>47</v>
       </c>
       <c r="I109" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -28771,7 +28879,7 @@
         <v>422</v>
       </c>
       <c r="E110" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F110" t="s">
         <v>0</v>
@@ -28783,7 +28891,7 @@
         <v>47</v>
       </c>
       <c r="I110" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="111" spans="1:9">
@@ -28797,10 +28905,10 @@
         <v>418</v>
       </c>
       <c r="D111" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E111" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F111" t="s">
         <v>0</v>
@@ -28812,7 +28920,7 @@
         <v>38</v>
       </c>
       <c r="I111" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="112" spans="1:9">
@@ -28826,10 +28934,10 @@
         <v>418</v>
       </c>
       <c r="D112" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E112" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F112" t="s">
         <v>0</v>
@@ -28841,7 +28949,7 @@
         <v>38</v>
       </c>
       <c r="I112" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -28855,10 +28963,10 @@
         <v>418</v>
       </c>
       <c r="D113" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E113" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F113" t="s">
         <v>0</v>
@@ -28870,7 +28978,7 @@
         <v>38</v>
       </c>
       <c r="I113" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -28884,10 +28992,10 @@
         <v>418</v>
       </c>
       <c r="D114" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E114" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F114" t="s">
         <v>0</v>
@@ -28899,7 +29007,7 @@
         <v>42</v>
       </c>
       <c r="I114" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -28913,10 +29021,10 @@
         <v>418</v>
       </c>
       <c r="D115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E115" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F115" t="s">
         <v>0</v>
@@ -28928,7 +29036,7 @@
         <v>39</v>
       </c>
       <c r="I115" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -28942,22 +29050,22 @@
         <v>414</v>
       </c>
       <c r="D116" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E116" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F116" t="s">
         <v>0</v>
       </c>
       <c r="G116" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H116">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I116" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -28971,22 +29079,22 @@
         <v>414</v>
       </c>
       <c r="D117" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E117" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F117" t="s">
         <v>0</v>
       </c>
       <c r="G117" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H117">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I117" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -29000,22 +29108,22 @@
         <v>414</v>
       </c>
       <c r="D118" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E118" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F118" t="s">
         <v>0</v>
       </c>
       <c r="G118" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H118">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I118" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -29029,22 +29137,22 @@
         <v>414</v>
       </c>
       <c r="D119" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E119" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F119" t="s">
         <v>0</v>
       </c>
       <c r="G119" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H119">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I119" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="120" spans="1:9">
@@ -29058,22 +29166,22 @@
         <v>414</v>
       </c>
       <c r="D120" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E120" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F120" t="s">
         <v>0</v>
       </c>
       <c r="G120" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H120">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I120" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -29087,22 +29195,22 @@
         <v>414</v>
       </c>
       <c r="D121" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E121" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F121" t="s">
         <v>0</v>
       </c>
       <c r="G121" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H121">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I121" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -29116,22 +29224,22 @@
         <v>414</v>
       </c>
       <c r="D122" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E122" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F122" t="s">
         <v>0</v>
       </c>
       <c r="G122" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H122">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I122" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="123" spans="1:9">
@@ -29145,22 +29253,22 @@
         <v>414</v>
       </c>
       <c r="D123" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E123" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F123" t="s">
         <v>0</v>
       </c>
       <c r="G123" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H123">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I123" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="124" spans="1:9">
@@ -29174,22 +29282,22 @@
         <v>414</v>
       </c>
       <c r="D124" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E124" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F124" t="s">
         <v>0</v>
       </c>
       <c r="G124" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H124">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I124" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="125" spans="1:9">
@@ -29203,22 +29311,22 @@
         <v>414</v>
       </c>
       <c r="D125" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E125" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F125" t="s">
         <v>0</v>
       </c>
       <c r="G125" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H125">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I125" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="126" spans="1:9">
@@ -29232,22 +29340,22 @@
         <v>414</v>
       </c>
       <c r="D126" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E126" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F126" t="s">
         <v>0</v>
       </c>
       <c r="G126" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H126">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I126" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="127" spans="1:9">
@@ -29261,22 +29369,22 @@
         <v>414</v>
       </c>
       <c r="D127" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E127" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F127" t="s">
         <v>0</v>
       </c>
       <c r="G127" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H127">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I127" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="128" spans="1:9">
@@ -29290,22 +29398,22 @@
         <v>414</v>
       </c>
       <c r="D128" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E128" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F128" t="s">
         <v>0</v>
       </c>
       <c r="G128" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H128">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I128" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="129" spans="1:9">
@@ -29319,22 +29427,22 @@
         <v>414</v>
       </c>
       <c r="D129" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E129" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F129" t="s">
         <v>0</v>
       </c>
       <c r="G129" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H129">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I129" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="130" spans="1:9">
@@ -29348,22 +29456,22 @@
         <v>414</v>
       </c>
       <c r="D130" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E130" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F130" t="s">
         <v>0</v>
       </c>
       <c r="G130" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H130">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I130" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="131" spans="1:9">
@@ -29377,22 +29485,22 @@
         <v>414</v>
       </c>
       <c r="D131" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E131" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F131" t="s">
         <v>0</v>
       </c>
       <c r="G131" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H131">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I131" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="132" spans="1:9">
@@ -29406,10 +29514,10 @@
         <v>419</v>
       </c>
       <c r="D132" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E132" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F132" t="s">
         <v>0</v>
@@ -29421,7 +29529,7 @@
         <v>41</v>
       </c>
       <c r="I132" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="133" spans="1:9">
@@ -29435,10 +29543,10 @@
         <v>419</v>
       </c>
       <c r="D133" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E133" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F133" t="s">
         <v>0</v>
@@ -29450,7 +29558,7 @@
         <v>40</v>
       </c>
       <c r="I133" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="134" spans="1:9">
@@ -29464,10 +29572,10 @@
         <v>419</v>
       </c>
       <c r="D134" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E134" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F134" t="s">
         <v>0</v>
@@ -29479,7 +29587,7 @@
         <v>45</v>
       </c>
       <c r="I134" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="135" spans="1:9">
@@ -29493,10 +29601,10 @@
         <v>419</v>
       </c>
       <c r="D135" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E135" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F135" t="s">
         <v>0</v>
@@ -29508,7 +29616,7 @@
         <v>45</v>
       </c>
       <c r="I135" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="136" spans="1:9">
@@ -29522,10 +29630,10 @@
         <v>406</v>
       </c>
       <c r="D136" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E136" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F136" t="s">
         <v>0</v>
@@ -29537,7 +29645,7 @@
         <v>46</v>
       </c>
       <c r="I136" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="137" spans="1:9">
@@ -29551,10 +29659,10 @@
         <v>406</v>
       </c>
       <c r="D137" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E137" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F137" t="s">
         <v>0</v>
@@ -29566,7 +29674,7 @@
         <v>46</v>
       </c>
       <c r="I137" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="138" spans="1:9">
@@ -29580,10 +29688,10 @@
         <v>406</v>
       </c>
       <c r="D138" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E138" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F138" t="s">
         <v>0</v>
@@ -29595,7 +29703,7 @@
         <v>46</v>
       </c>
       <c r="I138" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="139" spans="1:9">
@@ -29609,10 +29717,10 @@
         <v>406</v>
       </c>
       <c r="D139" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E139" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F139" t="s">
         <v>0</v>
@@ -29624,7 +29732,7 @@
         <v>46</v>
       </c>
       <c r="I139" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="140" spans="1:9">
@@ -29638,10 +29746,10 @@
         <v>406</v>
       </c>
       <c r="D140" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E140" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F140" t="s">
         <v>0</v>
@@ -29653,7 +29761,7 @@
         <v>46</v>
       </c>
       <c r="I140" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="141" spans="1:9">
@@ -29667,10 +29775,10 @@
         <v>406</v>
       </c>
       <c r="D141" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E141" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F141" t="s">
         <v>0</v>
@@ -29682,7 +29790,7 @@
         <v>46</v>
       </c>
       <c r="I141" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="142" spans="1:9">
@@ -29696,10 +29804,10 @@
         <v>406</v>
       </c>
       <c r="D142" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E142" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F142" t="s">
         <v>0</v>
@@ -29711,7 +29819,7 @@
         <v>46</v>
       </c>
       <c r="I142" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="143" spans="1:9">
@@ -29725,10 +29833,10 @@
         <v>406</v>
       </c>
       <c r="D143" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E143" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F143" t="s">
         <v>0</v>
@@ -29740,7 +29848,7 @@
         <v>46</v>
       </c>
       <c r="I143" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="144" spans="1:9">
@@ -29754,10 +29862,10 @@
         <v>406</v>
       </c>
       <c r="D144" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E144" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F144" t="s">
         <v>0</v>
@@ -29769,7 +29877,7 @@
         <v>46</v>
       </c>
       <c r="I144" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="145" spans="1:9">
@@ -29783,10 +29891,10 @@
         <v>406</v>
       </c>
       <c r="D145" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E145" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F145" t="s">
         <v>0</v>
@@ -29798,7 +29906,7 @@
         <v>46</v>
       </c>
       <c r="I145" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="146" spans="1:9">
@@ -29812,10 +29920,10 @@
         <v>406</v>
       </c>
       <c r="D146" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E146" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F146" t="s">
         <v>0</v>
@@ -29827,7 +29935,7 @@
         <v>46</v>
       </c>
       <c r="I146" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="147" spans="1:9">
@@ -29841,10 +29949,10 @@
         <v>406</v>
       </c>
       <c r="D147" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E147" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F147" t="s">
         <v>0</v>
@@ -29856,7 +29964,7 @@
         <v>46</v>
       </c>
       <c r="I147" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="148" spans="1:9">
@@ -29870,10 +29978,10 @@
         <v>406</v>
       </c>
       <c r="D148" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E148" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F148" t="s">
         <v>0</v>
@@ -29885,7 +29993,7 @@
         <v>46</v>
       </c>
       <c r="I148" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="149" spans="1:9">
@@ -29899,10 +30007,10 @@
         <v>406</v>
       </c>
       <c r="D149" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E149" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F149" t="s">
         <v>0</v>
@@ -29914,7 +30022,7 @@
         <v>46</v>
       </c>
       <c r="I149" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="150" spans="1:9">
@@ -29928,10 +30036,10 @@
         <v>406</v>
       </c>
       <c r="D150" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E150" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F150" t="s">
         <v>0</v>
@@ -29943,7 +30051,7 @@
         <v>46</v>
       </c>
       <c r="I150" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="151" spans="1:9">
@@ -29957,10 +30065,10 @@
         <v>406</v>
       </c>
       <c r="D151" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E151" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F151" t="s">
         <v>0</v>
@@ -29972,7 +30080,7 @@
         <v>46</v>
       </c>
       <c r="I151" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="152" spans="1:9">
@@ -29986,10 +30094,10 @@
         <v>406</v>
       </c>
       <c r="D152" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E152" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F152" t="s">
         <v>0</v>
@@ -30001,7 +30109,7 @@
         <v>46</v>
       </c>
       <c r="I152" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="153" spans="1:9">
@@ -30015,10 +30123,10 @@
         <v>406</v>
       </c>
       <c r="D153" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E153" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F153" t="s">
         <v>0</v>
@@ -30030,7 +30138,7 @@
         <v>46</v>
       </c>
       <c r="I153" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="154" spans="1:9">
@@ -30044,10 +30152,10 @@
         <v>406</v>
       </c>
       <c r="D154" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E154" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F154" t="s">
         <v>0</v>
@@ -30059,7 +30167,7 @@
         <v>46</v>
       </c>
       <c r="I154" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="155" spans="1:9">
@@ -30073,10 +30181,10 @@
         <v>406</v>
       </c>
       <c r="D155" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E155" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F155" t="s">
         <v>0</v>
@@ -30088,7 +30196,7 @@
         <v>46</v>
       </c>
       <c r="I155" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="156" spans="1:9">
@@ -30102,10 +30210,10 @@
         <v>406</v>
       </c>
       <c r="D156" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E156" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F156" t="s">
         <v>0</v>
@@ -30117,7 +30225,7 @@
         <v>46</v>
       </c>
       <c r="I156" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="157" spans="1:9">
@@ -30131,10 +30239,10 @@
         <v>406</v>
       </c>
       <c r="D157" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E157" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F157" t="s">
         <v>0</v>
@@ -30146,7 +30254,7 @@
         <v>46</v>
       </c>
       <c r="I157" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="158" spans="1:9">
@@ -30160,10 +30268,10 @@
         <v>420</v>
       </c>
       <c r="D158" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E158" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F158" t="s">
         <v>36</v>
@@ -30175,7 +30283,7 @@
         <v>11</v>
       </c>
       <c r="I158" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="159" spans="1:9">
@@ -30189,10 +30297,10 @@
         <v>420</v>
       </c>
       <c r="D159" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E159" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F159" t="s">
         <v>36</v>
@@ -30204,7 +30312,7 @@
         <v>11</v>
       </c>
       <c r="I159" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="160" spans="1:9">
@@ -30218,10 +30326,10 @@
         <v>420</v>
       </c>
       <c r="D160" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E160" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F160" t="s">
         <v>36</v>
@@ -30233,7 +30341,7 @@
         <v>11</v>
       </c>
       <c r="I160" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="161" spans="1:9">
@@ -30247,10 +30355,10 @@
         <v>410</v>
       </c>
       <c r="D161" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E161" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F161" t="s">
         <v>0</v>
@@ -30262,7 +30370,7 @@
         <v>48</v>
       </c>
       <c r="I161" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="162" spans="1:9">
@@ -30276,10 +30384,10 @@
         <v>410</v>
       </c>
       <c r="D162" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E162" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F162" t="s">
         <v>0</v>
@@ -30291,7 +30399,7 @@
         <v>47</v>
       </c>
       <c r="I162" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="163" spans="1:9">
@@ -30305,10 +30413,10 @@
         <v>410</v>
       </c>
       <c r="D163" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E163" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F163" t="s">
         <v>0</v>
@@ -30320,7 +30428,7 @@
         <v>47</v>
       </c>
       <c r="I163" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="164" spans="1:9">
@@ -30334,10 +30442,10 @@
         <v>410</v>
       </c>
       <c r="D164" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E164" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F164" t="s">
         <v>0</v>
@@ -30349,7 +30457,7 @@
         <v>48</v>
       </c>
       <c r="I164" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="165" spans="1:9">
@@ -30363,10 +30471,10 @@
         <v>409</v>
       </c>
       <c r="D165" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E165" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F165" t="s">
         <v>0</v>
@@ -30378,7 +30486,7 @@
         <v>48</v>
       </c>
       <c r="I165" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="166" spans="1:9">
@@ -30392,10 +30500,10 @@
         <v>409</v>
       </c>
       <c r="D166" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E166" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F166" t="s">
         <v>0</v>
@@ -30407,7 +30515,7 @@
         <v>47</v>
       </c>
       <c r="I166" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="167" spans="1:9">
@@ -30421,10 +30529,10 @@
         <v>409</v>
       </c>
       <c r="D167" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E167" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F167" t="s">
         <v>0</v>
@@ -30436,7 +30544,7 @@
         <v>47</v>
       </c>
       <c r="I167" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="168" spans="1:9">
@@ -30450,10 +30558,10 @@
         <v>409</v>
       </c>
       <c r="D168" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E168" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F168" t="s">
         <v>0</v>
@@ -30465,7 +30573,7 @@
         <v>48</v>
       </c>
       <c r="I168" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -30479,10 +30587,10 @@
         <v>418</v>
       </c>
       <c r="D169" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E169" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F169" t="s">
         <v>9</v>
@@ -30494,7 +30602,7 @@
         <v>37</v>
       </c>
       <c r="I169" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="170" spans="1:9">
@@ -30508,10 +30616,10 @@
         <v>418</v>
       </c>
       <c r="D170" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E170" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F170" t="s">
         <v>9</v>
@@ -30523,7 +30631,7 @@
         <v>37</v>
       </c>
       <c r="I170" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="171" spans="1:9">
@@ -30537,10 +30645,10 @@
         <v>418</v>
       </c>
       <c r="D171" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E171" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F171" t="s">
         <v>16</v>
@@ -30552,7 +30660,7 @@
         <v>30</v>
       </c>
       <c r="I171" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="172" spans="1:9">
@@ -30566,10 +30674,10 @@
         <v>418</v>
       </c>
       <c r="D172" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E172" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F172" t="s">
         <v>32</v>
@@ -30581,7 +30689,7 @@
         <v>14</v>
       </c>
       <c r="I172" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="173" spans="1:9">
@@ -30595,10 +30703,10 @@
         <v>418</v>
       </c>
       <c r="D173" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E173" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F173" t="s">
         <v>32</v>
@@ -30610,7 +30718,7 @@
         <v>14</v>
       </c>
       <c r="I173" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="174" spans="1:9">
@@ -30624,10 +30732,10 @@
         <v>418</v>
       </c>
       <c r="D174" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E174" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F174" t="s">
         <v>32</v>
@@ -30639,7 +30747,7 @@
         <v>14</v>
       </c>
       <c r="I174" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="175" spans="1:9">
@@ -30653,10 +30761,10 @@
         <v>421</v>
       </c>
       <c r="D175" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E175" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F175" t="s">
         <v>0</v>
@@ -30668,7 +30776,7 @@
         <v>47</v>
       </c>
       <c r="I175" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
   </sheetData>
@@ -30678,24 +30786,30 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
+        <v>553</v>
+      </c>
+      <c r="B1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C1" t="s">
+        <v>549</v>
+      </c>
+      <c r="D1" t="s">
         <v>550</v>
       </c>
-      <c r="B1" t="s">
-        <v>547</v>
-      </c>
-      <c r="C1" t="s">
-        <v>548</v>
-      </c>
-      <c r="D1" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>551</v>
+      </c>
+      <c r="F1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -30708,8 +30822,14 @@
       <c r="D2">
         <v>213.99</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2">
+        <v>105.67</v>
+      </c>
+      <c r="F2">
+        <v>108.32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -30722,8 +30842,14 @@
       <c r="D3">
         <v>242.36</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3">
+        <v>114.19</v>
+      </c>
+      <c r="F3">
+        <v>128.17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>2027</v>
       </c>
@@ -30736,8 +30862,14 @@
       <c r="D4">
         <v>317.32</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4">
+        <v>157.96</v>
+      </c>
+      <c r="F4">
+        <v>159.36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>2028</v>
       </c>
@@ -30750,8 +30882,14 @@
       <c r="D5">
         <v>319.81</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5">
+        <v>170.71</v>
+      </c>
+      <c r="F5">
+        <v>149.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>2029</v>
       </c>
@@ -30764,8 +30902,14 @@
       <c r="D6">
         <v>479.55</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6">
+        <v>170.05</v>
+      </c>
+      <c r="F6">
+        <v>309.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>2030</v>
       </c>
@@ -30778,8 +30922,14 @@
       <c r="D7">
         <v>435.68</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7">
+        <v>142.41</v>
+      </c>
+      <c r="F7">
+        <v>293.27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>2031</v>
       </c>
@@ -30792,8 +30942,14 @@
       <c r="D8">
         <v>428.23</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8">
+        <v>121.38</v>
+      </c>
+      <c r="F8">
+        <v>306.85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>2032</v>
       </c>
@@ -30806,8 +30962,14 @@
       <c r="D9">
         <v>382.51</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9">
+        <v>111.6</v>
+      </c>
+      <c r="F9">
+        <v>270.91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>2033</v>
       </c>
@@ -30820,8 +30982,14 @@
       <c r="D10">
         <v>289.71</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10">
+        <v>103.63</v>
+      </c>
+      <c r="F10">
+        <v>186.08</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>2034</v>
       </c>
@@ -30834,8 +31002,14 @@
       <c r="D11">
         <v>524.09</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11">
+        <v>107.51</v>
+      </c>
+      <c r="F11">
+        <v>416.58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>2035</v>
       </c>
@@ -30848,8 +31022,14 @@
       <c r="D12">
         <v>514.12</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="E12">
+        <v>86.01000000000001</v>
+      </c>
+      <c r="F12">
+        <v>428.11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>2036</v>
       </c>
@@ -30862,8 +31042,14 @@
       <c r="D13">
         <v>447.81</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="E13">
+        <v>68.56</v>
+      </c>
+      <c r="F13">
+        <v>379.25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>2037</v>
       </c>
@@ -30876,8 +31062,14 @@
       <c r="D14">
         <v>262.74</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="E14">
+        <v>57.19</v>
+      </c>
+      <c r="F14">
+        <v>205.55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>2038</v>
       </c>
@@ -30890,8 +31082,14 @@
       <c r="D15">
         <v>222.11</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="E15">
+        <v>53.89</v>
+      </c>
+      <c r="F15">
+        <v>168.22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>2039</v>
       </c>
@@ -30904,8 +31102,14 @@
       <c r="D16">
         <v>216.8</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16">
+        <v>51</v>
+      </c>
+      <c r="F16">
+        <v>165.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>2040</v>
       </c>
@@ -30918,8 +31122,14 @@
       <c r="D17">
         <v>227.42</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17">
+        <v>47.62</v>
+      </c>
+      <c r="F17">
+        <v>179.79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>2041</v>
       </c>
@@ -30932,8 +31142,14 @@
       <c r="D18">
         <v>192.41</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18">
+        <v>42.36</v>
+      </c>
+      <c r="F18">
+        <v>150.05</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>2042</v>
       </c>
@@ -30946,8 +31162,14 @@
       <c r="D19">
         <v>285.67</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19">
+        <v>39.21</v>
+      </c>
+      <c r="F19">
+        <v>246.46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>2043</v>
       </c>
@@ -30960,8 +31182,14 @@
       <c r="D20">
         <v>179.65</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20">
+        <v>33.49</v>
+      </c>
+      <c r="F20">
+        <v>146.16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>2044</v>
       </c>
@@ -30974,8 +31202,14 @@
       <c r="D21">
         <v>176.06</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21">
+        <v>31.2</v>
+      </c>
+      <c r="F21">
+        <v>144.85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>2045</v>
       </c>
@@ -30988,8 +31222,14 @@
       <c r="D22">
         <v>169.78</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22">
+        <v>28.81</v>
+      </c>
+      <c r="F22">
+        <v>140.97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>2046</v>
       </c>
@@ -31002,8 +31242,14 @@
       <c r="D23">
         <v>166.33</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23">
+        <v>26.66</v>
+      </c>
+      <c r="F23">
+        <v>139.67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>2047</v>
       </c>
@@ -31016,8 +31262,14 @@
       <c r="D24">
         <v>163.27</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24">
+        <v>24.55</v>
+      </c>
+      <c r="F24">
+        <v>138.72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>2048</v>
       </c>
@@ -31030,8 +31282,14 @@
       <c r="D25">
         <v>159.97</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25">
+        <v>22.52</v>
+      </c>
+      <c r="F25">
+        <v>137.45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>2049</v>
       </c>
@@ -31044,8 +31302,14 @@
       <c r="D26">
         <v>157.17</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26">
+        <v>20.35</v>
+      </c>
+      <c r="F26">
+        <v>136.82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>2050</v>
       </c>
@@ -31057,6 +31321,12 @@
       </c>
       <c r="D27">
         <v>154.73</v>
+      </c>
+      <c r="E27">
+        <v>18.32</v>
+      </c>
+      <c r="F27">
+        <v>136.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
History 2026Q3: exports/imports from NBU BOP_m file (API stops at August), September state budget (#74)
- loaders/nbu_files: BOP_m.xlsx monthly goods and services (sheet 1.1), shared month-header parser
- history: EXP_USD/IMP_USD/TRADE_BAL fill months the API lacks from the file
- B5_EXTERNAL: 2026Q3 exports/imports are facts once the history has all three months; Q4 keeps the model split
- B6_FISCAL: September 2026 Treasury deficit 99.3 bn UAH (cumulative 669.4 bn)
- refreshed data/history


Claude-Session: https://claude.ai/code/session_01UMkgsrK6QTEHqqRgiG741H

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/history/history.xlsx
+++ b/data/history/history.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1673" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1675" uniqueCount="554">
   <si>
     <t>2015Q1</t>
   </si>
@@ -1309,12 +1309,15 @@
     <t>НБУ API (Госстат); НБУ Wages_m.xlsx; пропуски из MacroStat</t>
   </si>
   <si>
+    <t>НБУ API и BOP_m.xlsx (платёжный баланс)</t>
+  </si>
+  <si>
+    <t>НБУ API (Казначейство)</t>
+  </si>
+  <si>
     <t>НБУ API (платёжный баланс)</t>
   </si>
   <si>
-    <t>НБУ API (Казначейство)</t>
-  </si>
-  <si>
     <t>Минфин (index.minfin.com.ua)</t>
   </si>
   <si>
@@ -1423,10 +1426,10 @@
     <t>Средняя месячная зарплата, среднее за квартал; 2010–2012 из файла НБУ Wages_m; оставшиеся пропуски 2022–2024 из квартальных данных Госстата (лист Salary)</t>
   </si>
   <si>
-    <t>Товары и услуги, кредит, сумма месяцев</t>
-  </si>
-  <si>
-    <t>Товары и услуги, дебет, сумма месяцев</t>
+    <t>Товары и услуги, кредит, сумма месяцев; последние месяцы до API из файла BOP_m</t>
+  </si>
+  <si>
+    <t>Товары и услуги, дебет, сумма месяцев; последние месяцы до API из файла BOP_m</t>
   </si>
   <si>
     <t>EXP_USD − IMP_USD</t>
@@ -1667,6 +1670,12 @@
   </si>
   <si>
     <t>external</t>
+  </si>
+  <si>
+    <t>external_interest</t>
+  </si>
+  <si>
+    <t>external_repayment</t>
   </si>
   <si>
     <t>year</t>
@@ -3156,6 +3165,9 @@
       <c r="AU8">
         <v>39.1</v>
       </c>
+      <c r="AV8">
+        <v>38.4</v>
+      </c>
     </row>
     <row r="9" spans="1:49">
       <c r="A9" t="s">
@@ -3303,7 +3315,7 @@
         <v>44.69044673913044</v>
       </c>
       <c r="AW9">
-        <v>44.9262125</v>
+        <v>45.02476</v>
       </c>
     </row>
     <row r="10" spans="1:49">
@@ -3452,7 +3464,7 @@
         <v>44.8624</v>
       </c>
       <c r="AW10">
-        <v>45.051</v>
+        <v>45.5293</v>
       </c>
     </row>
     <row r="11" spans="1:49">
@@ -3601,7 +3613,7 @@
         <v>16</v>
       </c>
       <c r="AW11">
-        <v>16</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="12" spans="1:49">
@@ -3746,6 +3758,9 @@
       <c r="AU12">
         <v>19.83115822623704</v>
       </c>
+      <c r="AV12">
+        <v>19.98829703300498</v>
+      </c>
     </row>
     <row r="13" spans="1:49">
       <c r="A13" t="s">
@@ -3889,6 +3904,9 @@
       <c r="AU13">
         <v>10.05497450613516</v>
       </c>
+      <c r="AV13">
+        <v>10.42740907713206</v>
+      </c>
     </row>
     <row r="14" spans="1:49">
       <c r="A14" t="s">
@@ -4347,6 +4365,9 @@
       <c r="AU17">
         <v>31419.66666666667</v>
       </c>
+      <c r="AV17">
+        <v>32429.33333333333</v>
+      </c>
     </row>
     <row r="18" spans="1:48">
       <c r="A18" t="s">
@@ -4490,6 +4511,9 @@
       <c r="AU18">
         <v>14387</v>
       </c>
+      <c r="AV18">
+        <v>12187</v>
+      </c>
     </row>
     <row r="19" spans="1:48">
       <c r="A19" t="s">
@@ -4633,6 +4657,9 @@
       <c r="AU19">
         <v>31814</v>
       </c>
+      <c r="AV19">
+        <v>32342</v>
+      </c>
     </row>
     <row r="20" spans="1:48">
       <c r="A20" t="s">
@@ -4775,6 +4802,9 @@
       </c>
       <c r="AU20">
         <v>-17427</v>
+      </c>
+      <c r="AV20">
+        <v>-20155</v>
       </c>
     </row>
     <row r="21" spans="1:48">
@@ -10995,6 +11025,9 @@
       <c r="AU36">
         <v>9.133333333333335</v>
       </c>
+      <c r="AV36">
+        <v>6.199999999999998</v>
+      </c>
     </row>
     <row r="37" spans="1:48">
       <c r="A37" t="s">
@@ -11281,6 +11314,9 @@
       <c r="AU38">
         <v>914723.0858999999</v>
       </c>
+      <c r="AV38">
+        <v>917327.197</v>
+      </c>
     </row>
     <row r="39" spans="1:48">
       <c r="A39" t="s">
@@ -11424,6 +11460,9 @@
       <c r="AU39">
         <v>4139259.1604</v>
       </c>
+      <c r="AV39">
+        <v>4195653.3797</v>
+      </c>
     </row>
     <row r="40" spans="1:48">
       <c r="A40" t="s">
@@ -11567,6 +11606,9 @@
       <c r="AU40">
         <v>15.55165556739514</v>
       </c>
+      <c r="AV40">
+        <v>17.75376782523249</v>
+      </c>
     </row>
     <row r="41" spans="1:48">
       <c r="A41" t="s">
@@ -11710,6 +11752,9 @@
       <c r="AU41">
         <v>29.2948390853322</v>
       </c>
+      <c r="AV41">
+        <v>29.08101818194272</v>
+      </c>
     </row>
     <row r="42" spans="1:48">
       <c r="A42" t="s">
@@ -11853,6 +11898,9 @@
       <c r="AU42">
         <v>10.38844073943397</v>
       </c>
+      <c r="AV42">
+        <v>10.31664473658278</v>
+      </c>
     </row>
     <row r="43" spans="1:48">
       <c r="A43" t="s">
@@ -13423,6 +13471,9 @@
       <c r="AU53">
         <v>9490799.6</v>
       </c>
+      <c r="AV53">
+        <v>9538348.800000001</v>
+      </c>
     </row>
     <row r="54" spans="1:48">
       <c r="A54" t="s">
@@ -14291,6 +14342,9 @@
       <c r="AU61">
         <v>5466.566666666667</v>
       </c>
+      <c r="AV61">
+        <v>5493.233333333334</v>
+      </c>
     </row>
     <row r="62" spans="1:48">
       <c r="A62" t="s">
@@ -16239,6 +16293,9 @@
       <c r="AU75">
         <v>14.7</v>
       </c>
+      <c r="AV75">
+        <v>13.6</v>
+      </c>
     </row>
     <row r="76" spans="1:48">
       <c r="A76" t="s">
@@ -16382,6 +16439,9 @@
       <c r="AU76">
         <v>9.9</v>
       </c>
+      <c r="AV76">
+        <v>3.4</v>
+      </c>
     </row>
     <row r="77" spans="1:48">
       <c r="A77" t="s">
@@ -17865,6 +17925,9 @@
       <c r="AU87">
         <v>6237.14266107</v>
       </c>
+      <c r="AV87">
+        <v>4467.46851447</v>
+      </c>
     </row>
     <row r="88" spans="1:48">
       <c r="A88" t="s">
@@ -18008,6 +18071,9 @@
       <c r="AU88">
         <v>2178.587996930001</v>
       </c>
+      <c r="AV88">
+        <v>1933.66236314</v>
+      </c>
     </row>
     <row r="89" spans="1:48">
       <c r="A89" t="s">
@@ -18151,6 +18217,9 @@
       <c r="AU89">
         <v>682.17082755</v>
       </c>
+      <c r="AV89">
+        <v>649.24482759</v>
+      </c>
     </row>
     <row r="90" spans="1:48">
       <c r="A90" t="s">
@@ -18294,6 +18363,9 @@
       <c r="AU90">
         <v>3323.99618793</v>
       </c>
+      <c r="AV90">
+        <v>3387.55877592</v>
+      </c>
     </row>
     <row r="91" spans="1:48">
       <c r="A91" t="s">
@@ -18437,6 +18509,9 @@
       <c r="AU91">
         <v>437.7822446900002</v>
       </c>
+      <c r="AV91">
+        <v>411.3390702800002</v>
+      </c>
     </row>
     <row r="92" spans="1:48">
       <c r="A92" t="s">
@@ -18580,6 +18655,9 @@
       <c r="AU92">
         <v>3451.173779139996</v>
       </c>
+      <c r="AV92">
+        <v>3109.25742917</v>
+      </c>
     </row>
     <row r="93" spans="1:48">
       <c r="A93" t="s">
@@ -18723,6 +18801,9 @@
       <c r="AU93">
         <v>533.57196893</v>
       </c>
+      <c r="AV93">
+        <v>509.52608051</v>
+      </c>
     </row>
     <row r="94" spans="1:48">
       <c r="A94" t="s">
@@ -18866,6 +18947,9 @@
       <c r="AU94">
         <v>339.2838354299998</v>
       </c>
+      <c r="AV94">
+        <v>311.4197745599998</v>
+      </c>
     </row>
     <row r="95" spans="1:48">
       <c r="A95" t="s">
@@ -19009,6 +19093,9 @@
       <c r="AU95">
         <v>196.9822311900001</v>
       </c>
+      <c r="AV95">
+        <v>188.10629171</v>
+      </c>
     </row>
     <row r="96" spans="1:48">
       <c r="A96" t="s">
@@ -19152,8 +19239,11 @@
       <c r="AU96">
         <v>966.9308393500008</v>
       </c>
-    </row>
-    <row r="97" spans="1:47">
+      <c r="AV96">
+        <v>1203.50340813</v>
+      </c>
+    </row>
+    <row r="97" spans="1:48">
       <c r="A97" t="s">
         <v>173</v>
       </c>
@@ -19295,8 +19385,11 @@
       <c r="AU97">
         <v>1227.76045312</v>
       </c>
-    </row>
-    <row r="98" spans="1:47">
+      <c r="AV97">
+        <v>714.61069847</v>
+      </c>
+    </row>
+    <row r="98" spans="1:48">
       <c r="A98" t="s">
         <v>174</v>
       </c>
@@ -19438,8 +19531,11 @@
       <c r="AU98">
         <v>1256.43277541</v>
       </c>
-    </row>
-    <row r="99" spans="1:47">
+      <c r="AV98">
+        <v>1208.091834829999</v>
+      </c>
+    </row>
+    <row r="99" spans="1:48">
       <c r="A99" t="s">
         <v>175</v>
       </c>
@@ -19581,8 +19677,11 @@
       <c r="AU99">
         <v>440.674090939998</v>
       </c>
-    </row>
-    <row r="100" spans="1:47">
+      <c r="AV99">
+        <v>413.133863630001</v>
+      </c>
+    </row>
+    <row r="100" spans="1:48">
       <c r="A100" t="s">
         <v>176</v>
       </c>
@@ -19724,8 +19823,11 @@
       <c r="AU100">
         <v>11435.77814950999</v>
       </c>
-    </row>
-    <row r="101" spans="1:47">
+      <c r="AV100">
+        <v>12807.93434983</v>
+      </c>
+    </row>
+    <row r="101" spans="1:48">
       <c r="A101" t="s">
         <v>177</v>
       </c>
@@ -19867,8 +19969,11 @@
       <c r="AU101">
         <v>435.9155225100026</v>
       </c>
-    </row>
-    <row r="102" spans="1:47">
+      <c r="AV101">
+        <v>602.5706533399989</v>
+      </c>
+    </row>
+    <row r="102" spans="1:48">
       <c r="A102" t="s">
         <v>178</v>
       </c>
@@ -20010,8 +20115,11 @@
       <c r="AU102">
         <v>2701.816436300007</v>
       </c>
-    </row>
-    <row r="103" spans="1:47">
+      <c r="AV102">
+        <v>1759.572064420003</v>
+      </c>
+    </row>
+    <row r="103" spans="1:48">
       <c r="A103" t="s">
         <v>179</v>
       </c>
@@ -20139,7 +20247,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="104" spans="1:47">
+    <row r="104" spans="1:48">
       <c r="A104" t="s">
         <v>180</v>
       </c>
@@ -20264,7 +20372,7 @@
         <v>243.6666666666667</v>
       </c>
     </row>
-    <row r="105" spans="1:47">
+    <row r="105" spans="1:48">
       <c r="A105" t="s">
         <v>181</v>
       </c>
@@ -20404,7 +20512,7 @@
         <v>1323.333333333333</v>
       </c>
     </row>
-    <row r="106" spans="1:47">
+    <row r="106" spans="1:48">
       <c r="A106" t="s">
         <v>182</v>
       </c>
@@ -20544,7 +20652,7 @@
         <v>463.3333333333333</v>
       </c>
     </row>
-    <row r="107" spans="1:47">
+    <row r="107" spans="1:48">
       <c r="A107" t="s">
         <v>183</v>
       </c>
@@ -20687,7 +20795,7 @@
         <v>1653117.9</v>
       </c>
     </row>
-    <row r="108" spans="1:47">
+    <row r="108" spans="1:48">
       <c r="A108" t="s">
         <v>184</v>
       </c>
@@ -20830,7 +20938,7 @@
         <v>237170.3</v>
       </c>
     </row>
-    <row r="109" spans="1:47">
+    <row r="109" spans="1:48">
       <c r="A109" t="s">
         <v>185</v>
       </c>
@@ -20973,7 +21081,7 @@
         <v>88222.2</v>
       </c>
     </row>
-    <row r="110" spans="1:47">
+    <row r="110" spans="1:48">
       <c r="A110" t="s">
         <v>186</v>
       </c>
@@ -21116,7 +21224,7 @@
         <v>78150.99999999999</v>
       </c>
     </row>
-    <row r="111" spans="1:47">
+    <row r="111" spans="1:48">
       <c r="A111" t="s">
         <v>187</v>
       </c>
@@ -21259,7 +21367,7 @@
         <v>170583</v>
       </c>
     </row>
-    <row r="112" spans="1:47">
+    <row r="112" spans="1:48">
       <c r="A112" t="s">
         <v>188</v>
       </c>
@@ -25651,7 +25759,7 @@
         <v>422</v>
       </c>
       <c r="E2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F2" t="s">
         <v>0</v>
@@ -25663,7 +25771,7 @@
         <v>46</v>
       </c>
       <c r="I2" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -25680,7 +25788,7 @@
         <v>422</v>
       </c>
       <c r="E3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F3" t="s">
         <v>0</v>
@@ -25692,7 +25800,7 @@
         <v>46</v>
       </c>
       <c r="I3" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -25709,7 +25817,7 @@
         <v>422</v>
       </c>
       <c r="E4" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F4" t="s">
         <v>0</v>
@@ -25721,7 +25829,7 @@
         <v>46</v>
       </c>
       <c r="I4" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -25738,7 +25846,7 @@
         <v>422</v>
       </c>
       <c r="E5" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
@@ -25750,7 +25858,7 @@
         <v>46</v>
       </c>
       <c r="I5" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -25767,7 +25875,7 @@
         <v>423</v>
       </c>
       <c r="E6" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F6" t="s">
         <v>0</v>
@@ -25779,7 +25887,7 @@
         <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -25796,7 +25904,7 @@
         <v>422</v>
       </c>
       <c r="E7" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F7" t="s">
         <v>0</v>
@@ -25808,7 +25916,7 @@
         <v>47</v>
       </c>
       <c r="I7" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -25825,19 +25933,19 @@
         <v>424</v>
       </c>
       <c r="E8" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F8" t="s">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H8">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I8" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -25854,7 +25962,7 @@
         <v>425</v>
       </c>
       <c r="E9" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F9" t="s">
         <v>0</v>
@@ -25866,7 +25974,7 @@
         <v>48</v>
       </c>
       <c r="I9" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -25883,7 +25991,7 @@
         <v>425</v>
       </c>
       <c r="E10" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F10" t="s">
         <v>0</v>
@@ -25895,7 +26003,7 @@
         <v>48</v>
       </c>
       <c r="I10" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -25912,7 +26020,7 @@
         <v>426</v>
       </c>
       <c r="E11" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F11" t="s">
         <v>0</v>
@@ -25924,7 +26032,7 @@
         <v>48</v>
       </c>
       <c r="I11" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -25941,19 +26049,19 @@
         <v>426</v>
       </c>
       <c r="E12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F12" t="s">
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H12">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I12" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -25970,19 +26078,19 @@
         <v>426</v>
       </c>
       <c r="E13" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F13" t="s">
         <v>0</v>
       </c>
       <c r="G13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H13">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I13" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -25999,7 +26107,7 @@
         <v>427</v>
       </c>
       <c r="E14" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F14" t="s">
         <v>0</v>
@@ -26011,7 +26119,7 @@
         <v>44</v>
       </c>
       <c r="I14" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -26028,7 +26136,7 @@
         <v>428</v>
       </c>
       <c r="E15" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F15" t="s">
         <v>0</v>
@@ -26040,7 +26148,7 @@
         <v>28</v>
       </c>
       <c r="I15" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -26057,7 +26165,7 @@
         <v>428</v>
       </c>
       <c r="E16" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F16" t="s">
         <v>0</v>
@@ -26069,7 +26177,7 @@
         <v>28</v>
       </c>
       <c r="I16" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -26086,19 +26194,19 @@
         <v>429</v>
       </c>
       <c r="E17" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F17" t="s">
         <v>0</v>
       </c>
       <c r="G17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H17">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I17" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -26115,19 +26223,19 @@
         <v>430</v>
       </c>
       <c r="E18" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F18" t="s">
         <v>0</v>
       </c>
       <c r="G18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H18">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I18" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -26144,19 +26252,19 @@
         <v>430</v>
       </c>
       <c r="E19" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F19" t="s">
         <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H19">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I19" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -26173,19 +26281,19 @@
         <v>423</v>
       </c>
       <c r="E20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F20" t="s">
         <v>0</v>
       </c>
       <c r="G20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H20">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I20" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -26202,7 +26310,7 @@
         <v>426</v>
       </c>
       <c r="E21" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F21" t="s">
         <v>0</v>
@@ -26214,7 +26322,7 @@
         <v>47</v>
       </c>
       <c r="I21" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -26231,7 +26339,7 @@
         <v>422</v>
       </c>
       <c r="E22" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F22" t="s">
         <v>0</v>
@@ -26243,7 +26351,7 @@
         <v>46</v>
       </c>
       <c r="I22" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -26260,7 +26368,7 @@
         <v>427</v>
       </c>
       <c r="E23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F23" t="s">
         <v>0</v>
@@ -26272,7 +26380,7 @@
         <v>28</v>
       </c>
       <c r="I23" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -26289,7 +26397,7 @@
         <v>431</v>
       </c>
       <c r="E24" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F24" t="s">
         <v>0</v>
@@ -26301,7 +26409,7 @@
         <v>46</v>
       </c>
       <c r="I24" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -26318,13 +26426,13 @@
         <v>423</v>
       </c>
       <c r="E25" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="I25" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -26338,10 +26446,10 @@
         <v>414</v>
       </c>
       <c r="D26" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E26" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F26" t="s">
         <v>0</v>
@@ -26353,7 +26461,7 @@
         <v>46</v>
       </c>
       <c r="I26" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -26370,13 +26478,13 @@
         <v>423</v>
       </c>
       <c r="E27" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="H27">
         <v>0</v>
       </c>
       <c r="I27" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -26390,10 +26498,10 @@
         <v>415</v>
       </c>
       <c r="D28" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E28" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F28" t="s">
         <v>0</v>
@@ -26405,7 +26513,7 @@
         <v>46</v>
       </c>
       <c r="I28" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -26422,7 +26530,7 @@
         <v>427</v>
       </c>
       <c r="E29" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F29" t="s">
         <v>0</v>
@@ -26434,7 +26542,7 @@
         <v>40</v>
       </c>
       <c r="I29" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -26448,10 +26556,10 @@
         <v>417</v>
       </c>
       <c r="D30" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E30" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F30" t="s">
         <v>12</v>
@@ -26463,7 +26571,7 @@
         <v>34</v>
       </c>
       <c r="I30" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -26480,7 +26588,7 @@
         <v>422</v>
       </c>
       <c r="E31" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F31" t="s">
         <v>0</v>
@@ -26492,7 +26600,7 @@
         <v>46</v>
       </c>
       <c r="I31" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -26509,7 +26617,7 @@
         <v>422</v>
       </c>
       <c r="E32" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F32" t="s">
         <v>0</v>
@@ -26521,7 +26629,7 @@
         <v>46</v>
       </c>
       <c r="I32" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -26538,7 +26646,7 @@
         <v>422</v>
       </c>
       <c r="E33" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F33" t="s">
         <v>0</v>
@@ -26550,7 +26658,7 @@
         <v>46</v>
       </c>
       <c r="I33" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -26567,7 +26675,7 @@
         <v>422</v>
       </c>
       <c r="E34" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F34" t="s">
         <v>0</v>
@@ -26579,7 +26687,7 @@
         <v>46</v>
       </c>
       <c r="I34" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -26596,7 +26704,7 @@
         <v>422</v>
       </c>
       <c r="E35" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F35" t="s">
         <v>0</v>
@@ -26608,7 +26716,7 @@
         <v>46</v>
       </c>
       <c r="I35" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -26625,7 +26733,7 @@
         <v>422</v>
       </c>
       <c r="E36" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F36" t="s">
         <v>0</v>
@@ -26637,7 +26745,7 @@
         <v>46</v>
       </c>
       <c r="I36" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -26654,7 +26762,7 @@
         <v>422</v>
       </c>
       <c r="E37" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F37" t="s">
         <v>0</v>
@@ -26666,7 +26774,7 @@
         <v>46</v>
       </c>
       <c r="I37" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -26683,7 +26791,7 @@
         <v>422</v>
       </c>
       <c r="E38" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F38" t="s">
         <v>0</v>
@@ -26695,7 +26803,7 @@
         <v>46</v>
       </c>
       <c r="I38" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -26712,7 +26820,7 @@
         <v>422</v>
       </c>
       <c r="E39" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F39" t="s">
         <v>0</v>
@@ -26724,7 +26832,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -26741,7 +26849,7 @@
         <v>422</v>
       </c>
       <c r="E40" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F40" t="s">
         <v>0</v>
@@ -26753,7 +26861,7 @@
         <v>46</v>
       </c>
       <c r="I40" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -26770,7 +26878,7 @@
         <v>422</v>
       </c>
       <c r="E41" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F41" t="s">
         <v>0</v>
@@ -26782,7 +26890,7 @@
         <v>46</v>
       </c>
       <c r="I41" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -26799,7 +26907,7 @@
         <v>422</v>
       </c>
       <c r="E42" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F42" t="s">
         <v>0</v>
@@ -26811,7 +26919,7 @@
         <v>46</v>
       </c>
       <c r="I42" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -26828,7 +26936,7 @@
         <v>422</v>
       </c>
       <c r="E43" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F43" t="s">
         <v>0</v>
@@ -26840,7 +26948,7 @@
         <v>46</v>
       </c>
       <c r="I43" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -26857,7 +26965,7 @@
         <v>422</v>
       </c>
       <c r="E44" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F44" t="s">
         <v>0</v>
@@ -26869,7 +26977,7 @@
         <v>46</v>
       </c>
       <c r="I44" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -26886,7 +26994,7 @@
         <v>422</v>
       </c>
       <c r="E45" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F45" t="s">
         <v>0</v>
@@ -26898,7 +27006,7 @@
         <v>46</v>
       </c>
       <c r="I45" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -26915,7 +27023,7 @@
         <v>422</v>
       </c>
       <c r="E46" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F46" t="s">
         <v>0</v>
@@ -26927,7 +27035,7 @@
         <v>46</v>
       </c>
       <c r="I46" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -26944,7 +27052,7 @@
         <v>422</v>
       </c>
       <c r="E47" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F47" t="s">
         <v>0</v>
@@ -26956,7 +27064,7 @@
         <v>46</v>
       </c>
       <c r="I47" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -26973,7 +27081,7 @@
         <v>422</v>
       </c>
       <c r="E48" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F48" t="s">
         <v>0</v>
@@ -26985,7 +27093,7 @@
         <v>46</v>
       </c>
       <c r="I48" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -27002,7 +27110,7 @@
         <v>422</v>
       </c>
       <c r="E49" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F49" t="s">
         <v>0</v>
@@ -27014,7 +27122,7 @@
         <v>46</v>
       </c>
       <c r="I49" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -27031,7 +27139,7 @@
         <v>422</v>
       </c>
       <c r="E50" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F50" t="s">
         <v>0</v>
@@ -27043,7 +27151,7 @@
         <v>46</v>
       </c>
       <c r="I50" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -27060,7 +27168,7 @@
         <v>422</v>
       </c>
       <c r="E51" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F51" t="s">
         <v>0</v>
@@ -27072,7 +27180,7 @@
         <v>46</v>
       </c>
       <c r="I51" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -27089,7 +27197,7 @@
         <v>422</v>
       </c>
       <c r="E52" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F52" t="s">
         <v>0</v>
@@ -27101,7 +27209,7 @@
         <v>46</v>
       </c>
       <c r="I52" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -27118,7 +27226,7 @@
         <v>422</v>
       </c>
       <c r="E53" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F53" t="s">
         <v>0</v>
@@ -27130,7 +27238,7 @@
         <v>46</v>
       </c>
       <c r="I53" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -27147,7 +27255,7 @@
         <v>422</v>
       </c>
       <c r="E54" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F54" t="s">
         <v>0</v>
@@ -27159,7 +27267,7 @@
         <v>46</v>
       </c>
       <c r="I54" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -27176,7 +27284,7 @@
         <v>422</v>
       </c>
       <c r="E55" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F55" t="s">
         <v>0</v>
@@ -27188,7 +27296,7 @@
         <v>46</v>
       </c>
       <c r="I55" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -27205,7 +27313,7 @@
         <v>422</v>
       </c>
       <c r="E56" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F56" t="s">
         <v>0</v>
@@ -27217,7 +27325,7 @@
         <v>46</v>
       </c>
       <c r="I56" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -27234,7 +27342,7 @@
         <v>422</v>
       </c>
       <c r="E57" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F57" t="s">
         <v>0</v>
@@ -27246,7 +27354,7 @@
         <v>46</v>
       </c>
       <c r="I57" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -27263,7 +27371,7 @@
         <v>422</v>
       </c>
       <c r="E58" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F58" t="s">
         <v>0</v>
@@ -27275,7 +27383,7 @@
         <v>46</v>
       </c>
       <c r="I58" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -27292,7 +27400,7 @@
         <v>422</v>
       </c>
       <c r="E59" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F59" t="s">
         <v>0</v>
@@ -27304,7 +27412,7 @@
         <v>46</v>
       </c>
       <c r="I59" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -27321,7 +27429,7 @@
         <v>422</v>
       </c>
       <c r="E60" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F60" t="s">
         <v>0</v>
@@ -27333,7 +27441,7 @@
         <v>46</v>
       </c>
       <c r="I60" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -27350,7 +27458,7 @@
         <v>422</v>
       </c>
       <c r="E61" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F61" t="s">
         <v>0</v>
@@ -27362,7 +27470,7 @@
         <v>46</v>
       </c>
       <c r="I61" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -27379,7 +27487,7 @@
         <v>422</v>
       </c>
       <c r="E62" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F62" t="s">
         <v>0</v>
@@ -27391,7 +27499,7 @@
         <v>47</v>
       </c>
       <c r="I62" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -27405,10 +27513,10 @@
         <v>418</v>
       </c>
       <c r="D63" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E63" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F63" t="s">
         <v>0</v>
@@ -27420,7 +27528,7 @@
         <v>47</v>
       </c>
       <c r="I63" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -27434,10 +27542,10 @@
         <v>418</v>
       </c>
       <c r="D64" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E64" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F64" t="s">
         <v>0</v>
@@ -27449,7 +27557,7 @@
         <v>46</v>
       </c>
       <c r="I64" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -27466,19 +27574,19 @@
         <v>422</v>
       </c>
       <c r="E65" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F65" t="s">
         <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H65">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I65" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -27495,7 +27603,7 @@
         <v>422</v>
       </c>
       <c r="E66" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F66" t="s">
         <v>0</v>
@@ -27507,7 +27615,7 @@
         <v>46</v>
       </c>
       <c r="I66" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -27524,19 +27632,19 @@
         <v>426</v>
       </c>
       <c r="E67" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F67" t="s">
         <v>0</v>
       </c>
       <c r="G67" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H67">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I67" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -27553,19 +27661,19 @@
         <v>426</v>
       </c>
       <c r="E68" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F68" t="s">
         <v>0</v>
       </c>
       <c r="G68" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H68">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I68" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -27582,19 +27690,19 @@
         <v>426</v>
       </c>
       <c r="E69" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F69" t="s">
         <v>0</v>
       </c>
       <c r="G69" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H69">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I69" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -27611,19 +27719,19 @@
         <v>426</v>
       </c>
       <c r="E70" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F70" t="s">
         <v>0</v>
       </c>
       <c r="G70" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H70">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I70" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -27640,19 +27748,19 @@
         <v>426</v>
       </c>
       <c r="E71" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F71" t="s">
         <v>0</v>
       </c>
       <c r="G71" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H71">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I71" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -27669,7 +27777,7 @@
         <v>431</v>
       </c>
       <c r="E72" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F72" t="s">
         <v>0</v>
@@ -27681,7 +27789,7 @@
         <v>46</v>
       </c>
       <c r="I72" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -27698,7 +27806,7 @@
         <v>431</v>
       </c>
       <c r="E73" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F73" t="s">
         <v>0</v>
@@ -27710,7 +27818,7 @@
         <v>44</v>
       </c>
       <c r="I73" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -27727,7 +27835,7 @@
         <v>431</v>
       </c>
       <c r="E74" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F74" t="s">
         <v>0</v>
@@ -27739,7 +27847,7 @@
         <v>46</v>
       </c>
       <c r="I74" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -27753,10 +27861,10 @@
         <v>414</v>
       </c>
       <c r="D75" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E75" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F75" t="s">
         <v>0</v>
@@ -27768,7 +27876,7 @@
         <v>46</v>
       </c>
       <c r="I75" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -27782,10 +27890,10 @@
         <v>414</v>
       </c>
       <c r="D76" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E76" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F76" t="s">
         <v>0</v>
@@ -27797,7 +27905,7 @@
         <v>46</v>
       </c>
       <c r="I76" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -27811,10 +27919,10 @@
         <v>414</v>
       </c>
       <c r="D77" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E77" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F77" t="s">
         <v>0</v>
@@ -27826,7 +27934,7 @@
         <v>46</v>
       </c>
       <c r="I77" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -27840,10 +27948,10 @@
         <v>414</v>
       </c>
       <c r="D78" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E78" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F78" t="s">
         <v>0</v>
@@ -27855,7 +27963,7 @@
         <v>46</v>
       </c>
       <c r="I78" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -27872,7 +27980,7 @@
         <v>426</v>
       </c>
       <c r="E79" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F79" t="s">
         <v>0</v>
@@ -27884,7 +27992,7 @@
         <v>47</v>
       </c>
       <c r="I79" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -27901,7 +28009,7 @@
         <v>426</v>
       </c>
       <c r="E80" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F80" t="s">
         <v>0</v>
@@ -27913,7 +28021,7 @@
         <v>46</v>
       </c>
       <c r="I80" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -27930,7 +28038,7 @@
         <v>426</v>
       </c>
       <c r="E81" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F81" t="s">
         <v>0</v>
@@ -27942,7 +28050,7 @@
         <v>46</v>
       </c>
       <c r="I81" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -27956,22 +28064,22 @@
         <v>406</v>
       </c>
       <c r="D82" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E82" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F82" t="s">
         <v>0</v>
       </c>
       <c r="G82" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H82">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I82" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -27985,10 +28093,10 @@
         <v>412</v>
       </c>
       <c r="D83" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E83" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F83" t="s">
         <v>0</v>
@@ -28000,7 +28108,7 @@
         <v>46</v>
       </c>
       <c r="I83" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -28014,10 +28122,10 @@
         <v>414</v>
       </c>
       <c r="D84" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E84" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F84" t="s">
         <v>28</v>
@@ -28029,7 +28137,7 @@
         <v>16</v>
       </c>
       <c r="I84" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -28043,10 +28151,10 @@
         <v>406</v>
       </c>
       <c r="D85" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E85" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F85" t="s">
         <v>28</v>
@@ -28058,7 +28166,7 @@
         <v>19</v>
       </c>
       <c r="I85" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="86" spans="1:9">
@@ -28072,10 +28180,10 @@
         <v>406</v>
       </c>
       <c r="D86" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E86" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F86" t="s">
         <v>28</v>
@@ -28087,7 +28195,7 @@
         <v>19</v>
       </c>
       <c r="I86" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -28101,10 +28209,10 @@
         <v>406</v>
       </c>
       <c r="D87" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E87" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F87" t="s">
         <v>0</v>
@@ -28116,7 +28224,7 @@
         <v>46</v>
       </c>
       <c r="I87" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -28130,10 +28238,10 @@
         <v>406</v>
       </c>
       <c r="D88" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E88" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F88" t="s">
         <v>0</v>
@@ -28145,7 +28253,7 @@
         <v>46</v>
       </c>
       <c r="I88" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -28159,10 +28267,10 @@
         <v>414</v>
       </c>
       <c r="D89" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E89" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F89" t="s">
         <v>0</v>
@@ -28174,7 +28282,7 @@
         <v>46</v>
       </c>
       <c r="I89" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -28188,22 +28296,22 @@
         <v>412</v>
       </c>
       <c r="D90" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="E90" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F90" t="s">
         <v>0</v>
       </c>
       <c r="G90" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H90">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I90" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -28217,10 +28325,10 @@
         <v>410</v>
       </c>
       <c r="D91" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E91" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F91" t="s">
         <v>0</v>
@@ -28232,7 +28340,7 @@
         <v>28</v>
       </c>
       <c r="I91" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -28249,7 +28357,7 @@
         <v>422</v>
       </c>
       <c r="E92" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F92" t="s">
         <v>0</v>
@@ -28261,7 +28369,7 @@
         <v>46</v>
       </c>
       <c r="I92" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -28278,7 +28386,7 @@
         <v>422</v>
       </c>
       <c r="E93" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F93" t="s">
         <v>0</v>
@@ -28290,7 +28398,7 @@
         <v>46</v>
       </c>
       <c r="I93" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -28307,7 +28415,7 @@
         <v>422</v>
       </c>
       <c r="E94" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F94" t="s">
         <v>0</v>
@@ -28319,7 +28427,7 @@
         <v>46</v>
       </c>
       <c r="I94" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -28336,7 +28444,7 @@
         <v>422</v>
       </c>
       <c r="E95" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F95" t="s">
         <v>0</v>
@@ -28348,7 +28456,7 @@
         <v>46</v>
       </c>
       <c r="I95" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -28365,7 +28473,7 @@
         <v>422</v>
       </c>
       <c r="E96" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F96" t="s">
         <v>0</v>
@@ -28377,7 +28485,7 @@
         <v>46</v>
       </c>
       <c r="I96" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -28394,7 +28502,7 @@
         <v>422</v>
       </c>
       <c r="E97" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F97" t="s">
         <v>0</v>
@@ -28406,7 +28514,7 @@
         <v>46</v>
       </c>
       <c r="I97" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -28423,7 +28531,7 @@
         <v>422</v>
       </c>
       <c r="E98" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F98" t="s">
         <v>0</v>
@@ -28435,7 +28543,7 @@
         <v>46</v>
       </c>
       <c r="I98" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -28452,7 +28560,7 @@
         <v>422</v>
       </c>
       <c r="E99" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F99" t="s">
         <v>0</v>
@@ -28464,7 +28572,7 @@
         <v>46</v>
       </c>
       <c r="I99" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="100" spans="1:9">
@@ -28481,7 +28589,7 @@
         <v>422</v>
       </c>
       <c r="E100" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="F100" t="s">
         <v>0</v>
@@ -28493,7 +28601,7 @@
         <v>46</v>
       </c>
       <c r="I100" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -28510,7 +28618,7 @@
         <v>422</v>
       </c>
       <c r="E101" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F101" t="s">
         <v>0</v>
@@ -28522,7 +28630,7 @@
         <v>46</v>
       </c>
       <c r="I101" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -28539,7 +28647,7 @@
         <v>422</v>
       </c>
       <c r="E102" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F102" t="s">
         <v>0</v>
@@ -28551,7 +28659,7 @@
         <v>46</v>
       </c>
       <c r="I102" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="103" spans="1:9">
@@ -28568,7 +28676,7 @@
         <v>422</v>
       </c>
       <c r="E103" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F103" t="s">
         <v>0</v>
@@ -28580,7 +28688,7 @@
         <v>46</v>
       </c>
       <c r="I103" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -28594,22 +28702,22 @@
         <v>418</v>
       </c>
       <c r="D104" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E104" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F104" t="s">
         <v>0</v>
       </c>
       <c r="G104" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H104">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I104" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -28623,22 +28731,22 @@
         <v>418</v>
       </c>
       <c r="D105" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E105" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F105" t="s">
         <v>0</v>
       </c>
       <c r="G105" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H105">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I105" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -28655,7 +28763,7 @@
         <v>422</v>
       </c>
       <c r="E106" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F106" t="s">
         <v>0</v>
@@ -28667,7 +28775,7 @@
         <v>47</v>
       </c>
       <c r="I106" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -28684,7 +28792,7 @@
         <v>422</v>
       </c>
       <c r="E107" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="F107" t="s">
         <v>0</v>
@@ -28696,7 +28804,7 @@
         <v>47</v>
       </c>
       <c r="I107" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -28713,7 +28821,7 @@
         <v>422</v>
       </c>
       <c r="E108" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F108" t="s">
         <v>0</v>
@@ -28725,7 +28833,7 @@
         <v>47</v>
       </c>
       <c r="I108" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -28742,7 +28850,7 @@
         <v>422</v>
       </c>
       <c r="E109" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F109" t="s">
         <v>0</v>
@@ -28754,7 +28862,7 @@
         <v>47</v>
       </c>
       <c r="I109" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -28771,7 +28879,7 @@
         <v>422</v>
       </c>
       <c r="E110" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F110" t="s">
         <v>0</v>
@@ -28783,7 +28891,7 @@
         <v>47</v>
       </c>
       <c r="I110" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="111" spans="1:9">
@@ -28797,10 +28905,10 @@
         <v>418</v>
       </c>
       <c r="D111" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E111" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F111" t="s">
         <v>0</v>
@@ -28812,7 +28920,7 @@
         <v>38</v>
       </c>
       <c r="I111" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="112" spans="1:9">
@@ -28826,10 +28934,10 @@
         <v>418</v>
       </c>
       <c r="D112" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E112" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F112" t="s">
         <v>0</v>
@@ -28841,7 +28949,7 @@
         <v>38</v>
       </c>
       <c r="I112" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -28855,10 +28963,10 @@
         <v>418</v>
       </c>
       <c r="D113" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E113" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F113" t="s">
         <v>0</v>
@@ -28870,7 +28978,7 @@
         <v>38</v>
       </c>
       <c r="I113" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -28884,10 +28992,10 @@
         <v>418</v>
       </c>
       <c r="D114" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E114" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F114" t="s">
         <v>0</v>
@@ -28899,7 +29007,7 @@
         <v>42</v>
       </c>
       <c r="I114" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -28913,10 +29021,10 @@
         <v>418</v>
       </c>
       <c r="D115" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E115" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F115" t="s">
         <v>0</v>
@@ -28928,7 +29036,7 @@
         <v>39</v>
       </c>
       <c r="I115" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -28942,22 +29050,22 @@
         <v>414</v>
       </c>
       <c r="D116" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E116" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F116" t="s">
         <v>0</v>
       </c>
       <c r="G116" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H116">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I116" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -28971,22 +29079,22 @@
         <v>414</v>
       </c>
       <c r="D117" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E117" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F117" t="s">
         <v>0</v>
       </c>
       <c r="G117" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H117">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I117" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -29000,22 +29108,22 @@
         <v>414</v>
       </c>
       <c r="D118" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E118" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F118" t="s">
         <v>0</v>
       </c>
       <c r="G118" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H118">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I118" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -29029,22 +29137,22 @@
         <v>414</v>
       </c>
       <c r="D119" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E119" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F119" t="s">
         <v>0</v>
       </c>
       <c r="G119" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H119">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I119" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="120" spans="1:9">
@@ -29058,22 +29166,22 @@
         <v>414</v>
       </c>
       <c r="D120" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E120" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F120" t="s">
         <v>0</v>
       </c>
       <c r="G120" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H120">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I120" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -29087,22 +29195,22 @@
         <v>414</v>
       </c>
       <c r="D121" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E121" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F121" t="s">
         <v>0</v>
       </c>
       <c r="G121" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H121">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I121" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -29116,22 +29224,22 @@
         <v>414</v>
       </c>
       <c r="D122" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E122" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F122" t="s">
         <v>0</v>
       </c>
       <c r="G122" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H122">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I122" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="123" spans="1:9">
@@ -29145,22 +29253,22 @@
         <v>414</v>
       </c>
       <c r="D123" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E123" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F123" t="s">
         <v>0</v>
       </c>
       <c r="G123" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H123">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I123" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="124" spans="1:9">
@@ -29174,22 +29282,22 @@
         <v>414</v>
       </c>
       <c r="D124" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E124" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F124" t="s">
         <v>0</v>
       </c>
       <c r="G124" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H124">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I124" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="125" spans="1:9">
@@ -29203,22 +29311,22 @@
         <v>414</v>
       </c>
       <c r="D125" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E125" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F125" t="s">
         <v>0</v>
       </c>
       <c r="G125" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H125">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I125" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="126" spans="1:9">
@@ -29232,22 +29340,22 @@
         <v>414</v>
       </c>
       <c r="D126" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E126" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F126" t="s">
         <v>0</v>
       </c>
       <c r="G126" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H126">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I126" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="127" spans="1:9">
@@ -29261,22 +29369,22 @@
         <v>414</v>
       </c>
       <c r="D127" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E127" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F127" t="s">
         <v>0</v>
       </c>
       <c r="G127" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H127">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I127" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="128" spans="1:9">
@@ -29290,22 +29398,22 @@
         <v>414</v>
       </c>
       <c r="D128" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E128" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F128" t="s">
         <v>0</v>
       </c>
       <c r="G128" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H128">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I128" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="129" spans="1:9">
@@ -29319,22 +29427,22 @@
         <v>414</v>
       </c>
       <c r="D129" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E129" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F129" t="s">
         <v>0</v>
       </c>
       <c r="G129" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H129">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I129" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="130" spans="1:9">
@@ -29348,22 +29456,22 @@
         <v>414</v>
       </c>
       <c r="D130" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E130" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F130" t="s">
         <v>0</v>
       </c>
       <c r="G130" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H130">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I130" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="131" spans="1:9">
@@ -29377,22 +29485,22 @@
         <v>414</v>
       </c>
       <c r="D131" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E131" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F131" t="s">
         <v>0</v>
       </c>
       <c r="G131" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H131">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I131" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="132" spans="1:9">
@@ -29406,10 +29514,10 @@
         <v>419</v>
       </c>
       <c r="D132" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E132" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F132" t="s">
         <v>0</v>
@@ -29421,7 +29529,7 @@
         <v>41</v>
       </c>
       <c r="I132" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="133" spans="1:9">
@@ -29435,10 +29543,10 @@
         <v>419</v>
       </c>
       <c r="D133" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E133" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F133" t="s">
         <v>0</v>
@@ -29450,7 +29558,7 @@
         <v>40</v>
       </c>
       <c r="I133" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="134" spans="1:9">
@@ -29464,10 +29572,10 @@
         <v>419</v>
       </c>
       <c r="D134" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E134" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F134" t="s">
         <v>0</v>
@@ -29479,7 +29587,7 @@
         <v>45</v>
       </c>
       <c r="I134" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="135" spans="1:9">
@@ -29493,10 +29601,10 @@
         <v>419</v>
       </c>
       <c r="D135" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E135" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F135" t="s">
         <v>0</v>
@@ -29508,7 +29616,7 @@
         <v>45</v>
       </c>
       <c r="I135" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="136" spans="1:9">
@@ -29522,10 +29630,10 @@
         <v>406</v>
       </c>
       <c r="D136" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E136" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F136" t="s">
         <v>0</v>
@@ -29537,7 +29645,7 @@
         <v>46</v>
       </c>
       <c r="I136" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="137" spans="1:9">
@@ -29551,10 +29659,10 @@
         <v>406</v>
       </c>
       <c r="D137" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E137" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F137" t="s">
         <v>0</v>
@@ -29566,7 +29674,7 @@
         <v>46</v>
       </c>
       <c r="I137" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="138" spans="1:9">
@@ -29580,10 +29688,10 @@
         <v>406</v>
       </c>
       <c r="D138" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E138" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F138" t="s">
         <v>0</v>
@@ -29595,7 +29703,7 @@
         <v>46</v>
       </c>
       <c r="I138" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="139" spans="1:9">
@@ -29609,10 +29717,10 @@
         <v>406</v>
       </c>
       <c r="D139" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E139" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F139" t="s">
         <v>0</v>
@@ -29624,7 +29732,7 @@
         <v>46</v>
       </c>
       <c r="I139" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="140" spans="1:9">
@@ -29638,10 +29746,10 @@
         <v>406</v>
       </c>
       <c r="D140" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E140" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F140" t="s">
         <v>0</v>
@@ -29653,7 +29761,7 @@
         <v>46</v>
       </c>
       <c r="I140" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="141" spans="1:9">
@@ -29667,10 +29775,10 @@
         <v>406</v>
       </c>
       <c r="D141" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E141" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F141" t="s">
         <v>0</v>
@@ -29682,7 +29790,7 @@
         <v>46</v>
       </c>
       <c r="I141" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="142" spans="1:9">
@@ -29696,10 +29804,10 @@
         <v>406</v>
       </c>
       <c r="D142" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E142" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F142" t="s">
         <v>0</v>
@@ -29711,7 +29819,7 @@
         <v>46</v>
       </c>
       <c r="I142" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="143" spans="1:9">
@@ -29725,10 +29833,10 @@
         <v>406</v>
       </c>
       <c r="D143" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E143" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F143" t="s">
         <v>0</v>
@@ -29740,7 +29848,7 @@
         <v>46</v>
       </c>
       <c r="I143" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="144" spans="1:9">
@@ -29754,10 +29862,10 @@
         <v>406</v>
       </c>
       <c r="D144" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E144" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F144" t="s">
         <v>0</v>
@@ -29769,7 +29877,7 @@
         <v>46</v>
       </c>
       <c r="I144" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="145" spans="1:9">
@@ -29783,10 +29891,10 @@
         <v>406</v>
       </c>
       <c r="D145" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E145" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F145" t="s">
         <v>0</v>
@@ -29798,7 +29906,7 @@
         <v>46</v>
       </c>
       <c r="I145" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="146" spans="1:9">
@@ -29812,10 +29920,10 @@
         <v>406</v>
       </c>
       <c r="D146" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E146" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F146" t="s">
         <v>0</v>
@@ -29827,7 +29935,7 @@
         <v>46</v>
       </c>
       <c r="I146" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="147" spans="1:9">
@@ -29841,10 +29949,10 @@
         <v>406</v>
       </c>
       <c r="D147" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E147" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F147" t="s">
         <v>0</v>
@@ -29856,7 +29964,7 @@
         <v>46</v>
       </c>
       <c r="I147" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="148" spans="1:9">
@@ -29870,10 +29978,10 @@
         <v>406</v>
       </c>
       <c r="D148" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E148" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F148" t="s">
         <v>0</v>
@@ -29885,7 +29993,7 @@
         <v>46</v>
       </c>
       <c r="I148" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="149" spans="1:9">
@@ -29899,10 +30007,10 @@
         <v>406</v>
       </c>
       <c r="D149" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E149" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F149" t="s">
         <v>0</v>
@@ -29914,7 +30022,7 @@
         <v>46</v>
       </c>
       <c r="I149" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="150" spans="1:9">
@@ -29928,10 +30036,10 @@
         <v>406</v>
       </c>
       <c r="D150" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E150" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F150" t="s">
         <v>0</v>
@@ -29943,7 +30051,7 @@
         <v>46</v>
       </c>
       <c r="I150" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="151" spans="1:9">
@@ -29957,10 +30065,10 @@
         <v>406</v>
       </c>
       <c r="D151" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E151" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F151" t="s">
         <v>0</v>
@@ -29972,7 +30080,7 @@
         <v>46</v>
       </c>
       <c r="I151" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="152" spans="1:9">
@@ -29986,10 +30094,10 @@
         <v>406</v>
       </c>
       <c r="D152" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E152" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F152" t="s">
         <v>0</v>
@@ -30001,7 +30109,7 @@
         <v>46</v>
       </c>
       <c r="I152" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="153" spans="1:9">
@@ -30015,10 +30123,10 @@
         <v>406</v>
       </c>
       <c r="D153" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E153" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F153" t="s">
         <v>0</v>
@@ -30030,7 +30138,7 @@
         <v>46</v>
       </c>
       <c r="I153" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="154" spans="1:9">
@@ -30044,10 +30152,10 @@
         <v>406</v>
       </c>
       <c r="D154" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E154" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F154" t="s">
         <v>0</v>
@@ -30059,7 +30167,7 @@
         <v>46</v>
       </c>
       <c r="I154" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="155" spans="1:9">
@@ -30073,10 +30181,10 @@
         <v>406</v>
       </c>
       <c r="D155" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E155" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F155" t="s">
         <v>0</v>
@@ -30088,7 +30196,7 @@
         <v>46</v>
       </c>
       <c r="I155" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="156" spans="1:9">
@@ -30102,10 +30210,10 @@
         <v>406</v>
       </c>
       <c r="D156" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E156" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F156" t="s">
         <v>0</v>
@@ -30117,7 +30225,7 @@
         <v>46</v>
       </c>
       <c r="I156" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="157" spans="1:9">
@@ -30131,10 +30239,10 @@
         <v>406</v>
       </c>
       <c r="D157" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E157" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F157" t="s">
         <v>0</v>
@@ -30146,7 +30254,7 @@
         <v>46</v>
       </c>
       <c r="I157" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="158" spans="1:9">
@@ -30160,10 +30268,10 @@
         <v>420</v>
       </c>
       <c r="D158" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E158" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F158" t="s">
         <v>36</v>
@@ -30175,7 +30283,7 @@
         <v>11</v>
       </c>
       <c r="I158" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="159" spans="1:9">
@@ -30189,10 +30297,10 @@
         <v>420</v>
       </c>
       <c r="D159" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E159" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F159" t="s">
         <v>36</v>
@@ -30204,7 +30312,7 @@
         <v>11</v>
       </c>
       <c r="I159" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="160" spans="1:9">
@@ -30218,10 +30326,10 @@
         <v>420</v>
       </c>
       <c r="D160" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E160" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F160" t="s">
         <v>36</v>
@@ -30233,7 +30341,7 @@
         <v>11</v>
       </c>
       <c r="I160" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="161" spans="1:9">
@@ -30247,10 +30355,10 @@
         <v>410</v>
       </c>
       <c r="D161" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E161" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F161" t="s">
         <v>0</v>
@@ -30262,7 +30370,7 @@
         <v>48</v>
       </c>
       <c r="I161" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="162" spans="1:9">
@@ -30276,10 +30384,10 @@
         <v>410</v>
       </c>
       <c r="D162" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E162" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F162" t="s">
         <v>0</v>
@@ -30291,7 +30399,7 @@
         <v>47</v>
       </c>
       <c r="I162" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="163" spans="1:9">
@@ -30305,10 +30413,10 @@
         <v>410</v>
       </c>
       <c r="D163" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E163" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F163" t="s">
         <v>0</v>
@@ -30320,7 +30428,7 @@
         <v>47</v>
       </c>
       <c r="I163" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="164" spans="1:9">
@@ -30334,10 +30442,10 @@
         <v>410</v>
       </c>
       <c r="D164" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E164" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F164" t="s">
         <v>0</v>
@@ -30349,7 +30457,7 @@
         <v>48</v>
       </c>
       <c r="I164" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="165" spans="1:9">
@@ -30363,10 +30471,10 @@
         <v>409</v>
       </c>
       <c r="D165" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E165" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F165" t="s">
         <v>0</v>
@@ -30378,7 +30486,7 @@
         <v>48</v>
       </c>
       <c r="I165" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="166" spans="1:9">
@@ -30392,10 +30500,10 @@
         <v>409</v>
       </c>
       <c r="D166" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E166" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F166" t="s">
         <v>0</v>
@@ -30407,7 +30515,7 @@
         <v>47</v>
       </c>
       <c r="I166" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="167" spans="1:9">
@@ -30421,10 +30529,10 @@
         <v>409</v>
       </c>
       <c r="D167" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E167" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F167" t="s">
         <v>0</v>
@@ -30436,7 +30544,7 @@
         <v>47</v>
       </c>
       <c r="I167" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="168" spans="1:9">
@@ -30450,10 +30558,10 @@
         <v>409</v>
       </c>
       <c r="D168" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E168" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F168" t="s">
         <v>0</v>
@@ -30465,7 +30573,7 @@
         <v>48</v>
       </c>
       <c r="I168" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -30479,10 +30587,10 @@
         <v>418</v>
       </c>
       <c r="D169" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E169" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F169" t="s">
         <v>9</v>
@@ -30494,7 +30602,7 @@
         <v>37</v>
       </c>
       <c r="I169" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="170" spans="1:9">
@@ -30508,10 +30616,10 @@
         <v>418</v>
       </c>
       <c r="D170" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E170" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F170" t="s">
         <v>9</v>
@@ -30523,7 +30631,7 @@
         <v>37</v>
       </c>
       <c r="I170" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="171" spans="1:9">
@@ -30537,10 +30645,10 @@
         <v>418</v>
       </c>
       <c r="D171" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E171" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F171" t="s">
         <v>16</v>
@@ -30552,7 +30660,7 @@
         <v>30</v>
       </c>
       <c r="I171" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="172" spans="1:9">
@@ -30566,10 +30674,10 @@
         <v>418</v>
       </c>
       <c r="D172" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E172" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F172" t="s">
         <v>32</v>
@@ -30581,7 +30689,7 @@
         <v>14</v>
       </c>
       <c r="I172" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="173" spans="1:9">
@@ -30595,10 +30703,10 @@
         <v>418</v>
       </c>
       <c r="D173" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E173" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F173" t="s">
         <v>32</v>
@@ -30610,7 +30718,7 @@
         <v>14</v>
       </c>
       <c r="I173" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="174" spans="1:9">
@@ -30624,10 +30732,10 @@
         <v>418</v>
       </c>
       <c r="D174" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E174" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F174" t="s">
         <v>32</v>
@@ -30639,7 +30747,7 @@
         <v>14</v>
       </c>
       <c r="I174" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="175" spans="1:9">
@@ -30653,10 +30761,10 @@
         <v>421</v>
       </c>
       <c r="D175" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E175" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F175" t="s">
         <v>0</v>
@@ -30668,7 +30776,7 @@
         <v>47</v>
       </c>
       <c r="I175" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
   </sheetData>
@@ -30678,24 +30786,30 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
+        <v>553</v>
+      </c>
+      <c r="B1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C1" t="s">
+        <v>549</v>
+      </c>
+      <c r="D1" t="s">
         <v>550</v>
       </c>
-      <c r="B1" t="s">
-        <v>547</v>
-      </c>
-      <c r="C1" t="s">
-        <v>548</v>
-      </c>
-      <c r="D1" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>551</v>
+      </c>
+      <c r="F1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -30708,8 +30822,14 @@
       <c r="D2">
         <v>213.99</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2">
+        <v>105.67</v>
+      </c>
+      <c r="F2">
+        <v>108.32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -30722,8 +30842,14 @@
       <c r="D3">
         <v>242.36</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3">
+        <v>114.19</v>
+      </c>
+      <c r="F3">
+        <v>128.17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>2027</v>
       </c>
@@ -30736,8 +30862,14 @@
       <c r="D4">
         <v>317.32</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4">
+        <v>157.96</v>
+      </c>
+      <c r="F4">
+        <v>159.36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>2028</v>
       </c>
@@ -30750,8 +30882,14 @@
       <c r="D5">
         <v>319.81</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5">
+        <v>170.71</v>
+      </c>
+      <c r="F5">
+        <v>149.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>2029</v>
       </c>
@@ -30764,8 +30902,14 @@
       <c r="D6">
         <v>479.55</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6">
+        <v>170.05</v>
+      </c>
+      <c r="F6">
+        <v>309.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>2030</v>
       </c>
@@ -30778,8 +30922,14 @@
       <c r="D7">
         <v>435.68</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7">
+        <v>142.41</v>
+      </c>
+      <c r="F7">
+        <v>293.27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>2031</v>
       </c>
@@ -30792,8 +30942,14 @@
       <c r="D8">
         <v>428.23</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8">
+        <v>121.38</v>
+      </c>
+      <c r="F8">
+        <v>306.85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>2032</v>
       </c>
@@ -30806,8 +30962,14 @@
       <c r="D9">
         <v>382.51</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9">
+        <v>111.6</v>
+      </c>
+      <c r="F9">
+        <v>270.91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>2033</v>
       </c>
@@ -30820,8 +30982,14 @@
       <c r="D10">
         <v>289.71</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10">
+        <v>103.63</v>
+      </c>
+      <c r="F10">
+        <v>186.08</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>2034</v>
       </c>
@@ -30834,8 +31002,14 @@
       <c r="D11">
         <v>524.09</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11">
+        <v>107.51</v>
+      </c>
+      <c r="F11">
+        <v>416.58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>2035</v>
       </c>
@@ -30848,8 +31022,14 @@
       <c r="D12">
         <v>514.12</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="E12">
+        <v>86.01000000000001</v>
+      </c>
+      <c r="F12">
+        <v>428.11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>2036</v>
       </c>
@@ -30862,8 +31042,14 @@
       <c r="D13">
         <v>447.81</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="E13">
+        <v>68.56</v>
+      </c>
+      <c r="F13">
+        <v>379.25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>2037</v>
       </c>
@@ -30876,8 +31062,14 @@
       <c r="D14">
         <v>262.74</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="E14">
+        <v>57.19</v>
+      </c>
+      <c r="F14">
+        <v>205.55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>2038</v>
       </c>
@@ -30890,8 +31082,14 @@
       <c r="D15">
         <v>222.11</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="E15">
+        <v>53.89</v>
+      </c>
+      <c r="F15">
+        <v>168.22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>2039</v>
       </c>
@@ -30904,8 +31102,14 @@
       <c r="D16">
         <v>216.8</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16">
+        <v>51</v>
+      </c>
+      <c r="F16">
+        <v>165.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>2040</v>
       </c>
@@ -30918,8 +31122,14 @@
       <c r="D17">
         <v>227.42</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17">
+        <v>47.62</v>
+      </c>
+      <c r="F17">
+        <v>179.79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>2041</v>
       </c>
@@ -30932,8 +31142,14 @@
       <c r="D18">
         <v>192.41</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18">
+        <v>42.36</v>
+      </c>
+      <c r="F18">
+        <v>150.05</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>2042</v>
       </c>
@@ -30946,8 +31162,14 @@
       <c r="D19">
         <v>285.67</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19">
+        <v>39.21</v>
+      </c>
+      <c r="F19">
+        <v>246.46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>2043</v>
       </c>
@@ -30960,8 +31182,14 @@
       <c r="D20">
         <v>179.65</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20">
+        <v>33.49</v>
+      </c>
+      <c r="F20">
+        <v>146.16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>2044</v>
       </c>
@@ -30974,8 +31202,14 @@
       <c r="D21">
         <v>176.06</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21">
+        <v>31.2</v>
+      </c>
+      <c r="F21">
+        <v>144.85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>2045</v>
       </c>
@@ -30988,8 +31222,14 @@
       <c r="D22">
         <v>169.78</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22">
+        <v>28.81</v>
+      </c>
+      <c r="F22">
+        <v>140.97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>2046</v>
       </c>
@@ -31002,8 +31242,14 @@
       <c r="D23">
         <v>166.33</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23">
+        <v>26.66</v>
+      </c>
+      <c r="F23">
+        <v>139.67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>2047</v>
       </c>
@@ -31016,8 +31262,14 @@
       <c r="D24">
         <v>163.27</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24">
+        <v>24.55</v>
+      </c>
+      <c r="F24">
+        <v>138.72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>2048</v>
       </c>
@@ -31030,8 +31282,14 @@
       <c r="D25">
         <v>159.97</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25">
+        <v>22.52</v>
+      </c>
+      <c r="F25">
+        <v>137.45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>2049</v>
       </c>
@@ -31044,8 +31302,14 @@
       <c r="D26">
         <v>157.17</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26">
+        <v>20.35</v>
+      </c>
+      <c r="F26">
+        <v>136.82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>2050</v>
       </c>
@@ -31057,6 +31321,12 @@
       </c>
       <c r="D27">
         <v>154.73</v>
+      </c>
+      <c r="E27">
+        <v>18.32</v>
+      </c>
+      <c r="F27">
+        <v>136.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>